<commit_message>
Add PiN results step2 hybrid for Somalia___SOM
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Somalia___SOM/PiN_step2_Somalia___SOM_1022_02PM.xlsx
+++ b/platform_PiN_output/Somalia___SOM/PiN_step2_Somalia___SOM_1022_02PM.xlsx
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>2456493</v>
+        <v>2575503</v>
       </c>
       <c r="F6" s="10" t="n"/>
       <c r="G6" s="10" t="n"/>
@@ -772,22 +772,22 @@
         <v>4184714</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>41.3</v>
+        <v>38.5</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>1728169</v>
+        <v>1609053</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>53.7</v>
+        <v>56.3</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>2249188</v>
+        <v>2355964</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>150916</v>
+        <v>163149</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>1.3</v>
@@ -796,10 +796,10 @@
         <v>56390</v>
       </c>
       <c r="S6" s="9" t="n">
-        <v>58.7</v>
+        <v>61.5</v>
       </c>
       <c r="T6" s="9" t="n">
-        <v>2456493</v>
+        <v>2575503</v>
       </c>
     </row>
     <row r="7">
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>2174428</v>
+        <v>2284091</v>
       </c>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
@@ -834,22 +834,22 @@
         <v>3818312</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>43.1</v>
+        <v>40.2</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>1643798</v>
+        <v>1534019</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>52.3</v>
+        <v>54.9</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>1997975</v>
+        <v>2096277</v>
       </c>
       <c r="O7" s="11" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>126600</v>
+        <v>137960</v>
       </c>
       <c r="Q7" s="11" t="n">
         <v>1.3</v>
@@ -858,10 +858,10 @@
         <v>49853</v>
       </c>
       <c r="S7" s="11" t="n">
-        <v>56.9</v>
+        <v>59.8</v>
       </c>
       <c r="T7" s="11" t="n">
-        <v>2174428</v>
+        <v>2284091</v>
       </c>
     </row>
     <row r="8">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>282065</v>
+        <v>291412</v>
       </c>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
@@ -896,22 +896,22 @@
         <v>366402</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>23</v>
+        <v>20.5</v>
       </c>
       <c r="L8" s="11" t="n">
-        <v>84371</v>
+        <v>75034</v>
       </c>
       <c r="M8" s="11" t="n">
-        <v>68.59999999999999</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="N8" s="11" t="n">
-        <v>251213</v>
+        <v>259686</v>
       </c>
       <c r="O8" s="11" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="P8" s="11" t="n">
-        <v>24315</v>
+        <v>25189</v>
       </c>
       <c r="Q8" s="11" t="n">
         <v>1.8</v>
@@ -920,10 +920,10 @@
         <v>6537</v>
       </c>
       <c r="S8" s="11" t="n">
-        <v>77</v>
+        <v>79.5</v>
       </c>
       <c r="T8" s="11" t="n">
-        <v>282065</v>
+        <v>291412</v>
       </c>
     </row>
     <row r="9">
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="E9" s="12" t="n">
-        <v>1194366</v>
+        <v>1252102</v>
       </c>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>1262128</v>
+        <v>1323401</v>
       </c>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="E11" s="13" t="n">
-        <v>188961</v>
+        <v>198116</v>
       </c>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="E12" s="13" t="n">
-        <v>245649</v>
+        <v>257550</v>
       </c>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
@@ -1181,22 +1181,22 @@
         <v>123388</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>62.8</v>
+        <v>60.1</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>77487</v>
+        <v>74156</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>33.4</v>
+        <v>35.5</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>41211</v>
+        <v>43803</v>
       </c>
       <c r="K6" s="25" t="n">
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="L6" s="25" t="n">
-        <v>4689</v>
+        <v>5429</v>
       </c>
       <c r="M6" s="26" t="n">
         <v>0</v>
@@ -1205,10 +1205,10 @@
         <v>0</v>
       </c>
       <c r="O6" s="27" t="n">
-        <v>37.2</v>
+        <v>39.9</v>
       </c>
       <c r="P6" s="27" t="n">
-        <v>45900</v>
+        <v>49232</v>
       </c>
       <c r="Q6" s="28" t="inlineStr">
         <is>
@@ -1230,10 +1230,10 @@
         <v>11059</v>
       </c>
       <c r="G7" s="23" t="n">
-        <v>64.90000000000001</v>
+        <v>64.5</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>7177</v>
+        <v>7133</v>
       </c>
       <c r="I7" s="24" t="n">
         <v>33.2</v>
@@ -1242,10 +1242,10 @@
         <v>3672</v>
       </c>
       <c r="K7" s="25" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="L7" s="25" t="n">
-        <v>210</v>
+        <v>265</v>
       </c>
       <c r="M7" s="26" t="n">
         <v>0</v>
@@ -1254,10 +1254,10 @@
         <v>0</v>
       </c>
       <c r="O7" s="27" t="n">
-        <v>35.1</v>
+        <v>35.6</v>
       </c>
       <c r="P7" s="27" t="n">
-        <v>3882</v>
+        <v>3937</v>
       </c>
       <c r="Q7" s="28" t="inlineStr">
         <is>
@@ -1279,16 +1279,16 @@
         <v>34157</v>
       </c>
       <c r="G8" s="23" t="n">
-        <v>53.4</v>
+        <v>52.9</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>18254</v>
+        <v>18066</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>42.7</v>
+        <v>43.2</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>14571</v>
+        <v>14742</v>
       </c>
       <c r="K8" s="25" t="n">
         <v>3</v>
@@ -1303,10 +1303,10 @@
         <v>307</v>
       </c>
       <c r="O8" s="27" t="n">
-        <v>46.6</v>
+        <v>47.1</v>
       </c>
       <c r="P8" s="27" t="n">
-        <v>15903</v>
+        <v>16074</v>
       </c>
       <c r="Q8" s="28" t="inlineStr">
         <is>
@@ -1328,22 +1328,22 @@
         <v>30984</v>
       </c>
       <c r="G9" s="23" t="n">
-        <v>42.1</v>
+        <v>41.6</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>13044</v>
+        <v>12889</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>50.5</v>
+        <v>51.6</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>15662</v>
+        <v>16003</v>
       </c>
       <c r="K9" s="25" t="n">
-        <v>6.3</v>
+        <v>5.7</v>
       </c>
       <c r="L9" s="25" t="n">
-        <v>1936</v>
+        <v>1766</v>
       </c>
       <c r="M9" s="26" t="n">
         <v>1.1</v>
@@ -1352,10 +1352,10 @@
         <v>341</v>
       </c>
       <c r="O9" s="27" t="n">
-        <v>57.9</v>
+        <v>58.5</v>
       </c>
       <c r="P9" s="27" t="n">
-        <v>17940</v>
+        <v>18110</v>
       </c>
       <c r="Q9" s="28" t="inlineStr">
         <is>
@@ -1377,22 +1377,22 @@
         <v>187972</v>
       </c>
       <c r="G10" s="23" t="n">
-        <v>38.7</v>
+        <v>37.1</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>72745</v>
+        <v>69738</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>55.2</v>
+        <v>54.8</v>
       </c>
       <c r="J10" s="24" t="n">
-        <v>103760</v>
+        <v>103009</v>
       </c>
       <c r="K10" s="25" t="n">
-        <v>6</v>
+        <v>8.1</v>
       </c>
       <c r="L10" s="25" t="n">
-        <v>11278</v>
+        <v>15226</v>
       </c>
       <c r="M10" s="26" t="n">
         <v>0</v>
@@ -1401,10 +1401,10 @@
         <v>0</v>
       </c>
       <c r="O10" s="27" t="n">
-        <v>61.2</v>
+        <v>62.9</v>
       </c>
       <c r="P10" s="27" t="n">
-        <v>115039</v>
+        <v>118234</v>
       </c>
       <c r="Q10" s="28" t="inlineStr">
         <is>
@@ -1426,16 +1426,16 @@
         <v>72088</v>
       </c>
       <c r="G11" s="23" t="n">
-        <v>62</v>
+        <v>61.3</v>
       </c>
       <c r="H11" s="23" t="n">
-        <v>44731</v>
+        <v>44190</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>36.5</v>
+        <v>37.2</v>
       </c>
       <c r="J11" s="24" t="n">
-        <v>26276</v>
+        <v>26817</v>
       </c>
       <c r="K11" s="25" t="n">
         <v>1.1</v>
@@ -1450,10 +1450,10 @@
         <v>288</v>
       </c>
       <c r="O11" s="27" t="n">
-        <v>38</v>
+        <v>38.7</v>
       </c>
       <c r="P11" s="27" t="n">
-        <v>27358</v>
+        <v>27898</v>
       </c>
       <c r="Q11" s="28" t="inlineStr">
         <is>
@@ -1475,22 +1475,22 @@
         <v>46731</v>
       </c>
       <c r="G12" s="23" t="n">
-        <v>52.7</v>
+        <v>51.6</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>24604</v>
+        <v>24137</v>
       </c>
       <c r="I12" s="24" t="n">
-        <v>40.7</v>
+        <v>41.9</v>
       </c>
       <c r="J12" s="24" t="n">
-        <v>19019</v>
+        <v>19580</v>
       </c>
       <c r="K12" s="25" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="L12" s="25" t="n">
-        <v>2991</v>
+        <v>2874</v>
       </c>
       <c r="M12" s="26" t="n">
         <v>0.2</v>
@@ -1499,10 +1499,10 @@
         <v>117</v>
       </c>
       <c r="O12" s="27" t="n">
-        <v>47.4</v>
+        <v>48.3</v>
       </c>
       <c r="P12" s="27" t="n">
-        <v>22127</v>
+        <v>22571</v>
       </c>
       <c r="Q12" s="28" t="inlineStr">
         <is>
@@ -1527,13 +1527,13 @@
         <v>22.2</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>11562</v>
+        <v>11555</v>
       </c>
       <c r="I13" s="24" t="n">
         <v>75.2</v>
       </c>
       <c r="J13" s="24" t="n">
-        <v>39172</v>
+        <v>39179</v>
       </c>
       <c r="K13" s="25" t="n">
         <v>2.6</v>
@@ -1551,7 +1551,7 @@
         <v>77.8</v>
       </c>
       <c r="P13" s="27" t="n">
-        <v>40558</v>
+        <v>40565</v>
       </c>
       <c r="Q13" s="28" t="inlineStr">
         <is>
@@ -1573,16 +1573,16 @@
         <v>68732</v>
       </c>
       <c r="G14" s="23" t="n">
-        <v>46.1</v>
+        <v>45.6</v>
       </c>
       <c r="H14" s="23" t="n">
-        <v>31669</v>
+        <v>31355</v>
       </c>
       <c r="I14" s="24" t="n">
-        <v>51.7</v>
+        <v>52.2</v>
       </c>
       <c r="J14" s="24" t="n">
-        <v>35532</v>
+        <v>35846</v>
       </c>
       <c r="K14" s="25" t="n">
         <v>1.3</v>
@@ -1597,10 +1597,10 @@
         <v>608</v>
       </c>
       <c r="O14" s="27" t="n">
-        <v>53.9</v>
+        <v>54.4</v>
       </c>
       <c r="P14" s="27" t="n">
-        <v>37057</v>
+        <v>37371</v>
       </c>
       <c r="Q14" s="28" t="inlineStr">
         <is>
@@ -1622,16 +1622,16 @@
         <v>19315</v>
       </c>
       <c r="G15" s="23" t="n">
-        <v>65.7</v>
+        <v>62.2</v>
       </c>
       <c r="H15" s="23" t="n">
-        <v>12690</v>
+        <v>12014</v>
       </c>
       <c r="I15" s="24" t="n">
-        <v>33.6</v>
+        <v>37.1</v>
       </c>
       <c r="J15" s="24" t="n">
-        <v>6490</v>
+        <v>7166</v>
       </c>
       <c r="K15" s="25" t="n">
         <v>0.3</v>
@@ -1646,10 +1646,10 @@
         <v>58</v>
       </c>
       <c r="O15" s="27" t="n">
-        <v>34.2</v>
+        <v>37.7</v>
       </c>
       <c r="P15" s="27" t="n">
-        <v>6606</v>
+        <v>7282</v>
       </c>
       <c r="Q15" s="28" t="inlineStr">
         <is>
@@ -1671,16 +1671,16 @@
         <v>65990</v>
       </c>
       <c r="G16" s="23" t="n">
-        <v>40.1</v>
+        <v>36.3</v>
       </c>
       <c r="H16" s="23" t="n">
-        <v>26435</v>
+        <v>23939</v>
       </c>
       <c r="I16" s="24" t="n">
-        <v>59.2</v>
+        <v>63</v>
       </c>
       <c r="J16" s="24" t="n">
-        <v>39048</v>
+        <v>41544</v>
       </c>
       <c r="K16" s="25" t="n">
         <v>0.8</v>
@@ -1695,10 +1695,10 @@
         <v>2</v>
       </c>
       <c r="O16" s="27" t="n">
-        <v>60</v>
+        <v>63.8</v>
       </c>
       <c r="P16" s="27" t="n">
-        <v>39588</v>
+        <v>42084</v>
       </c>
       <c r="Q16" s="28" t="inlineStr">
         <is>
@@ -1720,16 +1720,16 @@
         <v>149286</v>
       </c>
       <c r="G17" s="23" t="n">
-        <v>41.4</v>
+        <v>34.1</v>
       </c>
       <c r="H17" s="23" t="n">
-        <v>61819</v>
+        <v>50947</v>
       </c>
       <c r="I17" s="24" t="n">
-        <v>57.9</v>
+        <v>65.2</v>
       </c>
       <c r="J17" s="24" t="n">
-        <v>86508</v>
+        <v>97380</v>
       </c>
       <c r="K17" s="25" t="n">
         <v>0.1</v>
@@ -1744,10 +1744,10 @@
         <v>875</v>
       </c>
       <c r="O17" s="27" t="n">
-        <v>58.6</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="P17" s="27" t="n">
-        <v>87474</v>
+        <v>98346</v>
       </c>
       <c r="Q17" s="28" t="inlineStr">
         <is>
@@ -1769,16 +1769,16 @@
         <v>9550</v>
       </c>
       <c r="G18" s="23" t="n">
-        <v>52</v>
+        <v>45.5</v>
       </c>
       <c r="H18" s="23" t="n">
-        <v>4966</v>
+        <v>4345</v>
       </c>
       <c r="I18" s="24" t="n">
-        <v>47.5</v>
+        <v>54</v>
       </c>
       <c r="J18" s="24" t="n">
-        <v>4536</v>
+        <v>5157</v>
       </c>
       <c r="K18" s="25" t="n">
         <v>0</v>
@@ -1793,10 +1793,10 @@
         <v>48</v>
       </c>
       <c r="O18" s="27" t="n">
-        <v>48</v>
+        <v>54.5</v>
       </c>
       <c r="P18" s="27" t="n">
-        <v>4584</v>
+        <v>5205</v>
       </c>
       <c r="Q18" s="28" t="inlineStr">
         <is>
@@ -1818,22 +1818,22 @@
         <v>17619</v>
       </c>
       <c r="G19" s="23" t="n">
-        <v>56.1</v>
+        <v>42.4</v>
       </c>
       <c r="H19" s="23" t="n">
-        <v>9884</v>
+        <v>7471</v>
       </c>
       <c r="I19" s="24" t="n">
-        <v>40.9</v>
+        <v>55.3</v>
       </c>
       <c r="J19" s="24" t="n">
-        <v>7206</v>
+        <v>9743</v>
       </c>
       <c r="K19" s="25" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="L19" s="25" t="n">
-        <v>529</v>
+        <v>405</v>
       </c>
       <c r="M19" s="26" t="n">
         <v>0</v>
@@ -1842,10 +1842,10 @@
         <v>0</v>
       </c>
       <c r="O19" s="27" t="n">
-        <v>43.9</v>
+        <v>57.6</v>
       </c>
       <c r="P19" s="27" t="n">
-        <v>7735</v>
+        <v>10149</v>
       </c>
       <c r="Q19" s="28" t="inlineStr">
         <is>
@@ -1867,16 +1867,16 @@
         <v>18367</v>
       </c>
       <c r="G20" s="23" t="n">
-        <v>47.6</v>
+        <v>47.4</v>
       </c>
       <c r="H20" s="23" t="n">
-        <v>8752</v>
+        <v>8715</v>
       </c>
       <c r="I20" s="24" t="n">
-        <v>48.3</v>
+        <v>48.4</v>
       </c>
       <c r="J20" s="24" t="n">
-        <v>8862</v>
+        <v>8899</v>
       </c>
       <c r="K20" s="25" t="n">
         <v>4.1</v>
@@ -1891,10 +1891,10 @@
         <v>0</v>
       </c>
       <c r="O20" s="27" t="n">
-        <v>52.4</v>
+        <v>52.5</v>
       </c>
       <c r="P20" s="27" t="n">
-        <v>9615</v>
+        <v>9652</v>
       </c>
       <c r="Q20" s="28" t="inlineStr">
         <is>
@@ -1916,22 +1916,22 @@
         <v>31417</v>
       </c>
       <c r="G21" s="23" t="n">
-        <v>34.7</v>
+        <v>33.6</v>
       </c>
       <c r="H21" s="23" t="n">
-        <v>10910</v>
+        <v>10546</v>
       </c>
       <c r="I21" s="24" t="n">
-        <v>59.8</v>
+        <v>62.7</v>
       </c>
       <c r="J21" s="24" t="n">
-        <v>18776</v>
+        <v>19707</v>
       </c>
       <c r="K21" s="25" t="n">
-        <v>4.2</v>
+        <v>2.5</v>
       </c>
       <c r="L21" s="25" t="n">
-        <v>1330</v>
+        <v>791</v>
       </c>
       <c r="M21" s="26" t="n">
         <v>1.3</v>
@@ -1940,10 +1940,10 @@
         <v>401</v>
       </c>
       <c r="O21" s="27" t="n">
-        <v>65.3</v>
+        <v>66.5</v>
       </c>
       <c r="P21" s="27" t="n">
-        <v>20507</v>
+        <v>20900</v>
       </c>
       <c r="Q21" s="28" t="inlineStr">
         <is>
@@ -1968,13 +1968,13 @@
         <v>45.4</v>
       </c>
       <c r="H22" s="23" t="n">
-        <v>59082</v>
+        <v>59070</v>
       </c>
       <c r="I22" s="24" t="n">
         <v>54.1</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>70349</v>
+        <v>70360</v>
       </c>
       <c r="K22" s="25" t="n">
         <v>0</v>
@@ -1992,7 +1992,7 @@
         <v>54.6</v>
       </c>
       <c r="P22" s="27" t="n">
-        <v>71026</v>
+        <v>71038</v>
       </c>
       <c r="Q22" s="28" t="inlineStr">
         <is>
@@ -2014,16 +2014,16 @@
         <v>24113</v>
       </c>
       <c r="G23" s="23" t="n">
-        <v>37</v>
+        <v>29.5</v>
       </c>
       <c r="H23" s="23" t="n">
-        <v>8922</v>
+        <v>7113</v>
       </c>
       <c r="I23" s="24" t="n">
-        <v>62.7</v>
+        <v>70.2</v>
       </c>
       <c r="J23" s="24" t="n">
-        <v>15119</v>
+        <v>16927</v>
       </c>
       <c r="K23" s="25" t="n">
         <v>0</v>
@@ -2038,10 +2038,10 @@
         <v>72</v>
       </c>
       <c r="O23" s="27" t="n">
-        <v>63</v>
+        <v>70.5</v>
       </c>
       <c r="P23" s="27" t="n">
-        <v>15191</v>
+        <v>17000</v>
       </c>
       <c r="Q23" s="28" t="inlineStr">
         <is>
@@ -2063,22 +2063,22 @@
         <v>388705</v>
       </c>
       <c r="G24" s="23" t="n">
-        <v>49.3</v>
+        <v>47.1</v>
       </c>
       <c r="H24" s="23" t="n">
-        <v>191604</v>
+        <v>183232</v>
       </c>
       <c r="I24" s="24" t="n">
-        <v>43.9</v>
+        <v>47</v>
       </c>
       <c r="J24" s="24" t="n">
-        <v>170778</v>
+        <v>182632</v>
       </c>
       <c r="K24" s="25" t="n">
-        <v>3.2</v>
+        <v>2.3</v>
       </c>
       <c r="L24" s="25" t="n">
-        <v>12381</v>
+        <v>8910</v>
       </c>
       <c r="M24" s="26" t="n">
         <v>3.6</v>
@@ -2087,10 +2087,10 @@
         <v>13943</v>
       </c>
       <c r="O24" s="27" t="n">
-        <v>50.7</v>
+        <v>52.9</v>
       </c>
       <c r="P24" s="27" t="n">
-        <v>197101</v>
+        <v>205485</v>
       </c>
       <c r="Q24" s="28" t="inlineStr">
         <is>
@@ -2112,16 +2112,16 @@
         <v>74442</v>
       </c>
       <c r="G25" s="23" t="n">
-        <v>67.8</v>
+        <v>67.5</v>
       </c>
       <c r="H25" s="23" t="n">
-        <v>50509</v>
+        <v>50261</v>
       </c>
       <c r="I25" s="24" t="n">
-        <v>30.8</v>
+        <v>31.1</v>
       </c>
       <c r="J25" s="24" t="n">
-        <v>22937</v>
+        <v>23183</v>
       </c>
       <c r="K25" s="25" t="n">
         <v>1.2</v>
@@ -2136,10 +2136,10 @@
         <v>134</v>
       </c>
       <c r="O25" s="27" t="n">
-        <v>32.2</v>
+        <v>32.5</v>
       </c>
       <c r="P25" s="27" t="n">
-        <v>23937</v>
+        <v>24183</v>
       </c>
       <c r="Q25" s="28" t="inlineStr">
         <is>
@@ -2161,16 +2161,16 @@
         <v>93854</v>
       </c>
       <c r="G26" s="23" t="n">
-        <v>38</v>
+        <v>36.8</v>
       </c>
       <c r="H26" s="23" t="n">
-        <v>35645</v>
+        <v>34567</v>
       </c>
       <c r="I26" s="24" t="n">
-        <v>60.3</v>
+        <v>61.4</v>
       </c>
       <c r="J26" s="24" t="n">
-        <v>56568</v>
+        <v>57647</v>
       </c>
       <c r="K26" s="25" t="n">
         <v>1.4</v>
@@ -2185,10 +2185,10 @@
         <v>281</v>
       </c>
       <c r="O26" s="27" t="n">
-        <v>62</v>
+        <v>63.2</v>
       </c>
       <c r="P26" s="27" t="n">
-        <v>58209</v>
+        <v>59287</v>
       </c>
       <c r="Q26" s="28" t="inlineStr">
         <is>
@@ -2216,16 +2216,16 @@
         <v>17187</v>
       </c>
       <c r="I27" s="24" t="n">
-        <v>54.3</v>
+        <v>54.7</v>
       </c>
       <c r="J27" s="24" t="n">
-        <v>24367</v>
+        <v>24546</v>
       </c>
       <c r="K27" s="25" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="L27" s="25" t="n">
-        <v>3321</v>
+        <v>3141</v>
       </c>
       <c r="M27" s="26" t="n">
         <v>0</v>
@@ -2259,22 +2259,22 @@
         <v>129104</v>
       </c>
       <c r="G28" s="23" t="n">
-        <v>37</v>
+        <v>35.3</v>
       </c>
       <c r="H28" s="23" t="n">
-        <v>47714</v>
+        <v>45536</v>
       </c>
       <c r="I28" s="24" t="n">
-        <v>54.6</v>
+        <v>56.3</v>
       </c>
       <c r="J28" s="24" t="n">
-        <v>70536</v>
+        <v>72648</v>
       </c>
       <c r="K28" s="25" t="n">
         <v>7.6</v>
       </c>
       <c r="L28" s="25" t="n">
-        <v>9829</v>
+        <v>9830</v>
       </c>
       <c r="M28" s="26" t="n">
         <v>0.8</v>
@@ -2283,10 +2283,10 @@
         <v>1089</v>
       </c>
       <c r="O28" s="27" t="n">
-        <v>63.1</v>
+        <v>64.7</v>
       </c>
       <c r="P28" s="27" t="n">
-        <v>81454</v>
+        <v>83568</v>
       </c>
       <c r="Q28" s="28" t="inlineStr">
         <is>
@@ -2308,16 +2308,16 @@
         <v>103737</v>
       </c>
       <c r="G29" s="23" t="n">
-        <v>64.90000000000001</v>
+        <v>63.4</v>
       </c>
       <c r="H29" s="23" t="n">
-        <v>67360</v>
+        <v>65782</v>
       </c>
       <c r="I29" s="24" t="n">
-        <v>33.9</v>
+        <v>35.4</v>
       </c>
       <c r="J29" s="24" t="n">
-        <v>35118</v>
+        <v>36697</v>
       </c>
       <c r="K29" s="25" t="n">
         <v>1.1</v>
@@ -2332,10 +2332,10 @@
         <v>215</v>
       </c>
       <c r="O29" s="27" t="n">
-        <v>35.1</v>
+        <v>36.6</v>
       </c>
       <c r="P29" s="27" t="n">
-        <v>36428</v>
+        <v>38007</v>
       </c>
       <c r="Q29" s="28" t="inlineStr">
         <is>
@@ -2357,22 +2357,22 @@
         <v>68584</v>
       </c>
       <c r="G30" s="23" t="n">
-        <v>38.9</v>
+        <v>37</v>
       </c>
       <c r="H30" s="23" t="n">
-        <v>26662</v>
+        <v>25360</v>
       </c>
       <c r="I30" s="24" t="n">
-        <v>58</v>
+        <v>56.5</v>
       </c>
       <c r="J30" s="24" t="n">
-        <v>39766</v>
+        <v>38749</v>
       </c>
       <c r="K30" s="25" t="n">
-        <v>2.1</v>
+        <v>5.5</v>
       </c>
       <c r="L30" s="25" t="n">
-        <v>1467</v>
+        <v>3787</v>
       </c>
       <c r="M30" s="26" t="n">
         <v>1.1</v>
@@ -2381,10 +2381,10 @@
         <v>756</v>
       </c>
       <c r="O30" s="27" t="n">
-        <v>61.2</v>
+        <v>63.1</v>
       </c>
       <c r="P30" s="27" t="n">
-        <v>41990</v>
+        <v>43292</v>
       </c>
       <c r="Q30" s="28" t="inlineStr">
         <is>
@@ -2406,22 +2406,22 @@
         <v>135718</v>
       </c>
       <c r="G31" s="23" t="n">
-        <v>34.4</v>
+        <v>28.8</v>
       </c>
       <c r="H31" s="23" t="n">
-        <v>46753</v>
+        <v>39033</v>
       </c>
       <c r="I31" s="24" t="n">
-        <v>59.7</v>
+        <v>65.8</v>
       </c>
       <c r="J31" s="24" t="n">
-        <v>81074</v>
+        <v>89243</v>
       </c>
       <c r="K31" s="25" t="n">
-        <v>4.7</v>
+        <v>4.3</v>
       </c>
       <c r="L31" s="25" t="n">
-        <v>6371</v>
+        <v>5873</v>
       </c>
       <c r="M31" s="26" t="n">
         <v>1.1</v>
@@ -2430,10 +2430,10 @@
         <v>1521</v>
       </c>
       <c r="O31" s="27" t="n">
-        <v>65.59999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="P31" s="27" t="n">
-        <v>88966</v>
+        <v>96637</v>
       </c>
       <c r="Q31" s="28" t="inlineStr">
         <is>
@@ -2455,22 +2455,22 @@
         <v>33947</v>
       </c>
       <c r="G32" s="23" t="n">
-        <v>10.8</v>
+        <v>9.1</v>
       </c>
       <c r="H32" s="23" t="n">
-        <v>3669</v>
+        <v>3093</v>
       </c>
       <c r="I32" s="24" t="n">
-        <v>78.3</v>
+        <v>77.7</v>
       </c>
       <c r="J32" s="24" t="n">
-        <v>26579</v>
+        <v>26364</v>
       </c>
       <c r="K32" s="25" t="n">
-        <v>6.1</v>
+        <v>8.4</v>
       </c>
       <c r="L32" s="25" t="n">
-        <v>2063</v>
+        <v>2854</v>
       </c>
       <c r="M32" s="26" t="n">
         <v>4.9</v>
@@ -2479,10 +2479,10 @@
         <v>1647</v>
       </c>
       <c r="O32" s="27" t="n">
-        <v>89.2</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="P32" s="27" t="n">
-        <v>30289</v>
+        <v>30865</v>
       </c>
       <c r="Q32" s="28" t="inlineStr">
         <is>
@@ -2507,13 +2507,13 @@
         <v>23.4</v>
       </c>
       <c r="H33" s="23" t="n">
-        <v>5118</v>
+        <v>5115</v>
       </c>
       <c r="I33" s="24" t="n">
         <v>75.59999999999999</v>
       </c>
       <c r="J33" s="24" t="n">
-        <v>16504</v>
+        <v>16507</v>
       </c>
       <c r="K33" s="25" t="n">
         <v>1</v>
@@ -2531,7 +2531,7 @@
         <v>76.59999999999999</v>
       </c>
       <c r="P33" s="27" t="n">
-        <v>16735</v>
+        <v>16738</v>
       </c>
       <c r="Q33" s="28" t="inlineStr">
         <is>
@@ -2556,13 +2556,13 @@
         <v>1.9</v>
       </c>
       <c r="H34" s="23" t="n">
-        <v>2214</v>
+        <v>2143</v>
       </c>
       <c r="I34" s="24" t="n">
-        <v>94.40000000000001</v>
+        <v>94.5</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>107748</v>
+        <v>107819</v>
       </c>
       <c r="K34" s="25" t="n">
         <v>2.8</v>
@@ -2577,10 +2577,10 @@
         <v>983</v>
       </c>
       <c r="O34" s="27" t="n">
-        <v>98.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="P34" s="27" t="n">
-        <v>111973</v>
+        <v>112043</v>
       </c>
       <c r="Q34" s="28" t="inlineStr">
         <is>
@@ -2651,16 +2651,16 @@
         <v>55853</v>
       </c>
       <c r="G36" s="23" t="n">
-        <v>76</v>
+        <v>75.8</v>
       </c>
       <c r="H36" s="23" t="n">
-        <v>42426</v>
+        <v>42310</v>
       </c>
       <c r="I36" s="24" t="n">
-        <v>16.9</v>
+        <v>17.1</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>9448</v>
+        <v>9564</v>
       </c>
       <c r="K36" s="25" t="n">
         <v>6.2</v>
@@ -2675,10 +2675,10 @@
         <v>474</v>
       </c>
       <c r="O36" s="27" t="n">
-        <v>24</v>
+        <v>24.2</v>
       </c>
       <c r="P36" s="27" t="n">
-        <v>13382</v>
+        <v>13498</v>
       </c>
       <c r="Q36" s="28" t="inlineStr">
         <is>
@@ -2700,22 +2700,22 @@
         <v>638</v>
       </c>
       <c r="G37" s="23" t="n">
-        <v>20.3</v>
+        <v>19.6</v>
       </c>
       <c r="H37" s="23" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="I37" s="24" t="n">
-        <v>78.3</v>
+        <v>79.7</v>
       </c>
       <c r="J37" s="24" t="n">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="K37" s="25" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="L37" s="25" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M37" s="26" t="n">
         <v>0.7</v>
@@ -2724,10 +2724,10 @@
         <v>4</v>
       </c>
       <c r="O37" s="27" t="n">
-        <v>79.7</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="P37" s="27" t="n">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="Q37" s="28" t="inlineStr">
         <is>
@@ -2847,22 +2847,22 @@
         <v>120511</v>
       </c>
       <c r="G40" s="23" t="n">
-        <v>56.5</v>
+        <v>55.9</v>
       </c>
       <c r="H40" s="23" t="n">
-        <v>68044</v>
+        <v>67381</v>
       </c>
       <c r="I40" s="24" t="n">
-        <v>43.2</v>
+        <v>43.6</v>
       </c>
       <c r="J40" s="24" t="n">
-        <v>52106</v>
+        <v>52588</v>
       </c>
       <c r="K40" s="25" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="L40" s="25" t="n">
-        <v>181</v>
+        <v>361</v>
       </c>
       <c r="M40" s="26" t="n">
         <v>0.2</v>
@@ -2871,10 +2871,10 @@
         <v>181</v>
       </c>
       <c r="O40" s="27" t="n">
-        <v>43.5</v>
+        <v>44.1</v>
       </c>
       <c r="P40" s="27" t="n">
-        <v>52467</v>
+        <v>53130</v>
       </c>
       <c r="Q40" s="28" t="inlineStr">
         <is>
@@ -2896,16 +2896,16 @@
         <v>148330</v>
       </c>
       <c r="G41" s="23" t="n">
-        <v>12.9</v>
+        <v>10.7</v>
       </c>
       <c r="H41" s="23" t="n">
-        <v>19195</v>
+        <v>15934</v>
       </c>
       <c r="I41" s="24" t="n">
-        <v>81.8</v>
+        <v>84</v>
       </c>
       <c r="J41" s="24" t="n">
-        <v>121277</v>
+        <v>124544</v>
       </c>
       <c r="K41" s="25" t="n">
         <v>2.1</v>
@@ -2920,10 +2920,10 @@
         <v>4676</v>
       </c>
       <c r="O41" s="27" t="n">
-        <v>87.09999999999999</v>
+        <v>89.3</v>
       </c>
       <c r="P41" s="27" t="n">
-        <v>129129</v>
+        <v>132396</v>
       </c>
       <c r="Q41" s="28" t="inlineStr">
         <is>
@@ -2945,16 +2945,16 @@
         <v>13582</v>
       </c>
       <c r="G42" s="23" t="n">
-        <v>84.8</v>
+        <v>83.8</v>
       </c>
       <c r="H42" s="23" t="n">
-        <v>11517</v>
+        <v>11381</v>
       </c>
       <c r="I42" s="24" t="n">
-        <v>15.2</v>
+        <v>16.2</v>
       </c>
       <c r="J42" s="24" t="n">
-        <v>2064</v>
+        <v>2200</v>
       </c>
       <c r="K42" s="25" t="n">
         <v>0</v>
@@ -2969,10 +2969,10 @@
         <v>0</v>
       </c>
       <c r="O42" s="27" t="n">
-        <v>15.2</v>
+        <v>16.2</v>
       </c>
       <c r="P42" s="27" t="n">
-        <v>2064</v>
+        <v>2200</v>
       </c>
       <c r="Q42" s="28" t="inlineStr">
         <is>
@@ -2994,22 +2994,22 @@
         <v>29215</v>
       </c>
       <c r="G43" s="23" t="n">
-        <v>36.9</v>
+        <v>36.1</v>
       </c>
       <c r="H43" s="23" t="n">
-        <v>10780</v>
+        <v>10547</v>
       </c>
       <c r="I43" s="24" t="n">
-        <v>60.2</v>
+        <v>60.6</v>
       </c>
       <c r="J43" s="24" t="n">
-        <v>17588</v>
+        <v>17704</v>
       </c>
       <c r="K43" s="25" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="L43" s="25" t="n">
-        <v>234</v>
+        <v>351</v>
       </c>
       <c r="M43" s="26" t="n">
         <v>2.1</v>
@@ -3018,10 +3018,10 @@
         <v>614</v>
       </c>
       <c r="O43" s="27" t="n">
-        <v>63.1</v>
+        <v>63.9</v>
       </c>
       <c r="P43" s="27" t="n">
-        <v>18435</v>
+        <v>18669</v>
       </c>
       <c r="Q43" s="28" t="inlineStr">
         <is>
@@ -3043,22 +3043,22 @@
         <v>42673</v>
       </c>
       <c r="G44" s="23" t="n">
-        <v>48.7</v>
+        <v>17.5</v>
       </c>
       <c r="H44" s="23" t="n">
-        <v>20784</v>
+        <v>7487</v>
       </c>
       <c r="I44" s="24" t="n">
-        <v>48.6</v>
+        <v>80.3</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>20724</v>
+        <v>34275</v>
       </c>
       <c r="K44" s="25" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="L44" s="25" t="n">
-        <v>609</v>
+        <v>311</v>
       </c>
       <c r="M44" s="26" t="n">
         <v>1.3</v>
@@ -3067,10 +3067,10 @@
         <v>556</v>
       </c>
       <c r="O44" s="27" t="n">
-        <v>51.3</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="P44" s="27" t="n">
-        <v>21889</v>
+        <v>35143</v>
       </c>
       <c r="Q44" s="28" t="inlineStr">
         <is>
@@ -3092,22 +3092,22 @@
         <v>352402</v>
       </c>
       <c r="G45" s="23" t="n">
-        <v>49.7</v>
+        <v>41.9</v>
       </c>
       <c r="H45" s="23" t="n">
-        <v>175234</v>
+        <v>147516</v>
       </c>
       <c r="I45" s="24" t="n">
-        <v>44.4</v>
+        <v>52.2</v>
       </c>
       <c r="J45" s="24" t="n">
-        <v>156482</v>
+        <v>184123</v>
       </c>
       <c r="K45" s="25" t="n">
         <v>4.7</v>
       </c>
       <c r="L45" s="25" t="n">
-        <v>16614</v>
+        <v>16535</v>
       </c>
       <c r="M45" s="26" t="n">
         <v>1.2</v>
@@ -3116,10 +3116,10 @@
         <v>4229</v>
       </c>
       <c r="O45" s="27" t="n">
-        <v>50.3</v>
+        <v>58.1</v>
       </c>
       <c r="P45" s="27" t="n">
-        <v>177325</v>
+        <v>204886</v>
       </c>
       <c r="Q45" s="28" t="inlineStr">
         <is>
@@ -3141,16 +3141,16 @@
         <v>78051</v>
       </c>
       <c r="G46" s="23" t="n">
-        <v>15.7</v>
+        <v>15.4</v>
       </c>
       <c r="H46" s="23" t="n">
-        <v>12256</v>
+        <v>12025</v>
       </c>
       <c r="I46" s="24" t="n">
-        <v>75.8</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="J46" s="24" t="n">
-        <v>59151</v>
+        <v>59383</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>5.4</v>
@@ -3165,10 +3165,10 @@
         <v>2392</v>
       </c>
       <c r="O46" s="27" t="n">
-        <v>84.3</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="P46" s="27" t="n">
-        <v>65795</v>
+        <v>66026</v>
       </c>
       <c r="Q46" s="28" t="inlineStr">
         <is>
@@ -3190,16 +3190,16 @@
         <v>72194</v>
       </c>
       <c r="G47" s="23" t="n">
-        <v>24.6</v>
+        <v>24</v>
       </c>
       <c r="H47" s="23" t="n">
-        <v>17761</v>
+        <v>17315</v>
       </c>
       <c r="I47" s="24" t="n">
-        <v>63.4</v>
+        <v>64</v>
       </c>
       <c r="J47" s="24" t="n">
-        <v>45790</v>
+        <v>46237</v>
       </c>
       <c r="K47" s="25" t="n">
         <v>9.800000000000001</v>
@@ -3214,10 +3214,10 @@
         <v>1572</v>
       </c>
       <c r="O47" s="27" t="n">
-        <v>75.40000000000001</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="P47" s="27" t="n">
-        <v>54460</v>
+        <v>54906</v>
       </c>
       <c r="Q47" s="28" t="inlineStr">
         <is>
@@ -3239,22 +3239,22 @@
         <v>61647</v>
       </c>
       <c r="G48" s="23" t="n">
-        <v>51.6</v>
+        <v>39.8</v>
       </c>
       <c r="H48" s="23" t="n">
-        <v>31809</v>
+        <v>24525</v>
       </c>
       <c r="I48" s="24" t="n">
-        <v>34.3</v>
+        <v>46.2</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>21126</v>
+        <v>28454</v>
       </c>
       <c r="K48" s="25" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="L48" s="25" t="n">
-        <v>6219</v>
+        <v>6175</v>
       </c>
       <c r="M48" s="26" t="n">
         <v>4</v>
@@ -3263,10 +3263,10 @@
         <v>2462</v>
       </c>
       <c r="O48" s="27" t="n">
-        <v>48.4</v>
+        <v>60.2</v>
       </c>
       <c r="P48" s="27" t="n">
-        <v>29807</v>
+        <v>37091</v>
       </c>
       <c r="Q48" s="28" t="inlineStr">
         <is>
@@ -3288,22 +3288,22 @@
         <v>16004</v>
       </c>
       <c r="G49" s="23" t="n">
-        <v>48.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H49" s="23" t="n">
-        <v>7778</v>
+        <v>1472</v>
       </c>
       <c r="I49" s="24" t="n">
-        <v>47.7</v>
+        <v>86.2</v>
       </c>
       <c r="J49" s="24" t="n">
-        <v>7634</v>
+        <v>13795</v>
       </c>
       <c r="K49" s="25" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L49" s="25" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="M49" s="26" t="n">
         <v>3.7</v>
@@ -3312,10 +3312,10 @@
         <v>592</v>
       </c>
       <c r="O49" s="27" t="n">
-        <v>51.4</v>
+        <v>90.8</v>
       </c>
       <c r="P49" s="27" t="n">
-        <v>8226</v>
+        <v>14531</v>
       </c>
       <c r="Q49" s="28" t="inlineStr">
         <is>
@@ -3337,16 +3337,16 @@
         <v>34876</v>
       </c>
       <c r="G50" s="23" t="n">
-        <v>63</v>
+        <v>61.5</v>
       </c>
       <c r="H50" s="23" t="n">
-        <v>21989</v>
+        <v>21433</v>
       </c>
       <c r="I50" s="24" t="n">
-        <v>36.8</v>
+        <v>38.4</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>12833</v>
+        <v>13389</v>
       </c>
       <c r="K50" s="25" t="n">
         <v>0.2</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="O50" s="27" t="n">
-        <v>37</v>
+        <v>38.5</v>
       </c>
       <c r="P50" s="27" t="n">
-        <v>12887</v>
+        <v>13443</v>
       </c>
       <c r="Q50" s="28" t="inlineStr">
         <is>
@@ -3386,22 +3386,22 @@
         <v>18832</v>
       </c>
       <c r="G51" s="23" t="n">
-        <v>13.7</v>
+        <v>4.1</v>
       </c>
       <c r="H51" s="23" t="n">
-        <v>2575</v>
+        <v>779</v>
       </c>
       <c r="I51" s="24" t="n">
-        <v>71.40000000000001</v>
+        <v>80.2</v>
       </c>
       <c r="J51" s="24" t="n">
-        <v>13444</v>
+        <v>15098</v>
       </c>
       <c r="K51" s="25" t="n">
-        <v>12.6</v>
+        <v>13.5</v>
       </c>
       <c r="L51" s="25" t="n">
-        <v>2377</v>
+        <v>2536</v>
       </c>
       <c r="M51" s="26" t="n">
         <v>2.2</v>
@@ -3410,10 +3410,10 @@
         <v>419</v>
       </c>
       <c r="O51" s="27" t="n">
-        <v>86.2</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="P51" s="27" t="n">
-        <v>16240</v>
+        <v>18053</v>
       </c>
       <c r="Q51" s="28" t="inlineStr">
         <is>
@@ -3435,22 +3435,22 @@
         <v>74863</v>
       </c>
       <c r="G52" s="23" t="n">
-        <v>38.3</v>
+        <v>36.7</v>
       </c>
       <c r="H52" s="23" t="n">
-        <v>28655</v>
+        <v>27449</v>
       </c>
       <c r="I52" s="24" t="n">
-        <v>57.5</v>
+        <v>58.1</v>
       </c>
       <c r="J52" s="24" t="n">
-        <v>43014</v>
+        <v>43525</v>
       </c>
       <c r="K52" s="25" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="L52" s="25" t="n">
-        <v>2274</v>
+        <v>2942</v>
       </c>
       <c r="M52" s="26" t="n">
         <v>1.2</v>
@@ -3459,10 +3459,10 @@
         <v>935</v>
       </c>
       <c r="O52" s="27" t="n">
-        <v>61.7</v>
+        <v>63.3</v>
       </c>
       <c r="P52" s="27" t="n">
-        <v>46223</v>
+        <v>47402</v>
       </c>
       <c r="Q52" s="28" t="inlineStr">
         <is>
@@ -3484,16 +3484,16 @@
         <v>37406</v>
       </c>
       <c r="G53" s="23" t="n">
-        <v>28.2</v>
+        <v>25.1</v>
       </c>
       <c r="H53" s="23" t="n">
-        <v>10551</v>
+        <v>9408</v>
       </c>
       <c r="I53" s="24" t="n">
-        <v>62.4</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J53" s="24" t="n">
-        <v>23336</v>
+        <v>24466</v>
       </c>
       <c r="K53" s="25" t="n">
         <v>5</v>
@@ -3508,10 +3508,10 @@
         <v>1653</v>
       </c>
       <c r="O53" s="27" t="n">
-        <v>71.8</v>
+        <v>74.8</v>
       </c>
       <c r="P53" s="27" t="n">
-        <v>26851</v>
+        <v>27980</v>
       </c>
       <c r="Q53" s="28" t="inlineStr">
         <is>
@@ -3533,16 +3533,16 @@
         <v>19699</v>
       </c>
       <c r="G54" s="23" t="n">
-        <v>18.1</v>
+        <v>14.9</v>
       </c>
       <c r="H54" s="23" t="n">
-        <v>3574</v>
+        <v>2942</v>
       </c>
       <c r="I54" s="24" t="n">
-        <v>66</v>
+        <v>69.2</v>
       </c>
       <c r="J54" s="24" t="n">
-        <v>13011</v>
+        <v>13633</v>
       </c>
       <c r="K54" s="25" t="n">
         <v>14.1</v>
@@ -3557,10 +3557,10 @@
         <v>346</v>
       </c>
       <c r="O54" s="27" t="n">
-        <v>81.90000000000001</v>
+        <v>85</v>
       </c>
       <c r="P54" s="27" t="n">
-        <v>16125</v>
+        <v>16748</v>
       </c>
       <c r="Q54" s="28" t="inlineStr">
         <is>
@@ -3582,22 +3582,22 @@
         <v>70546</v>
       </c>
       <c r="G55" s="23" t="n">
-        <v>31.8</v>
+        <v>29.7</v>
       </c>
       <c r="H55" s="23" t="n">
-        <v>22411</v>
+        <v>20962</v>
       </c>
       <c r="I55" s="24" t="n">
-        <v>53.8</v>
+        <v>52.5</v>
       </c>
       <c r="J55" s="24" t="n">
-        <v>37977</v>
+        <v>37072</v>
       </c>
       <c r="K55" s="25" t="n">
-        <v>13</v>
+        <v>16.3</v>
       </c>
       <c r="L55" s="25" t="n">
-        <v>9142</v>
+        <v>11465</v>
       </c>
       <c r="M55" s="26" t="n">
         <v>1.4</v>
@@ -3606,10 +3606,10 @@
         <v>1017</v>
       </c>
       <c r="O55" s="27" t="n">
-        <v>68.2</v>
+        <v>70.2</v>
       </c>
       <c r="P55" s="27" t="n">
-        <v>48136</v>
+        <v>49554</v>
       </c>
       <c r="Q55" s="28" t="inlineStr">
         <is>
@@ -3631,16 +3631,16 @@
         <v>47485</v>
       </c>
       <c r="G56" s="23" t="n">
-        <v>18.6</v>
+        <v>17.9</v>
       </c>
       <c r="H56" s="23" t="n">
-        <v>8836</v>
+        <v>8480</v>
       </c>
       <c r="I56" s="24" t="n">
-        <v>79.7</v>
+        <v>80.5</v>
       </c>
       <c r="J56" s="24" t="n">
-        <v>37859</v>
+        <v>38215</v>
       </c>
       <c r="K56" s="25" t="n">
         <v>1.5</v>
@@ -3655,10 +3655,10 @@
         <v>90</v>
       </c>
       <c r="O56" s="27" t="n">
-        <v>81.40000000000001</v>
+        <v>82.2</v>
       </c>
       <c r="P56" s="27" t="n">
-        <v>38668</v>
+        <v>39024</v>
       </c>
       <c r="Q56" s="28" t="inlineStr">
         <is>
@@ -3680,22 +3680,22 @@
         <v>44224</v>
       </c>
       <c r="G57" s="23" t="n">
-        <v>49.7</v>
+        <v>47.7</v>
       </c>
       <c r="H57" s="23" t="n">
-        <v>21977</v>
+        <v>21093</v>
       </c>
       <c r="I57" s="24" t="n">
-        <v>31.1</v>
+        <v>32.3</v>
       </c>
       <c r="J57" s="24" t="n">
-        <v>13742</v>
+        <v>14279</v>
       </c>
       <c r="K57" s="25" t="n">
-        <v>13.8</v>
+        <v>14.6</v>
       </c>
       <c r="L57" s="25" t="n">
-        <v>6090</v>
+        <v>6445</v>
       </c>
       <c r="M57" s="26" t="n">
         <v>5.5</v>
@@ -3704,14 +3704,14 @@
         <v>2414</v>
       </c>
       <c r="O57" s="27" t="n">
-        <v>50.3</v>
+        <v>52.3</v>
       </c>
       <c r="P57" s="27" t="n">
-        <v>22247</v>
+        <v>23138</v>
       </c>
       <c r="Q57" s="28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3729,22 +3729,22 @@
         <v>57479</v>
       </c>
       <c r="G58" s="23" t="n">
-        <v>80.2</v>
+        <v>78.8</v>
       </c>
       <c r="H58" s="23" t="n">
-        <v>46089</v>
+        <v>45291</v>
       </c>
       <c r="I58" s="24" t="n">
-        <v>15.3</v>
+        <v>16.7</v>
       </c>
       <c r="J58" s="24" t="n">
-        <v>8821</v>
+        <v>9604</v>
       </c>
       <c r="K58" s="25" t="n">
         <v>4</v>
       </c>
       <c r="L58" s="25" t="n">
-        <v>2296</v>
+        <v>2310</v>
       </c>
       <c r="M58" s="26" t="n">
         <v>0.5</v>
@@ -3753,14 +3753,14 @@
         <v>273</v>
       </c>
       <c r="O58" s="27" t="n">
-        <v>19.8</v>
+        <v>21.2</v>
       </c>
       <c r="P58" s="27" t="n">
-        <v>11390</v>
+        <v>12187</v>
       </c>
       <c r="Q58" s="28" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -3778,10 +3778,10 @@
         <v>7176</v>
       </c>
       <c r="G59" s="23" t="n">
-        <v>56.7</v>
+        <v>55</v>
       </c>
       <c r="H59" s="23" t="n">
-        <v>4069</v>
+        <v>3947</v>
       </c>
       <c r="I59" s="24" t="n">
         <v>40</v>
@@ -3790,10 +3790,10 @@
         <v>2870</v>
       </c>
       <c r="K59" s="25" t="n">
-        <v>1.7</v>
+        <v>3.3</v>
       </c>
       <c r="L59" s="25" t="n">
-        <v>122</v>
+        <v>237</v>
       </c>
       <c r="M59" s="26" t="n">
         <v>1.7</v>
@@ -3802,10 +3802,10 @@
         <v>122</v>
       </c>
       <c r="O59" s="27" t="n">
-        <v>43.4</v>
+        <v>45</v>
       </c>
       <c r="P59" s="27" t="n">
-        <v>3114</v>
+        <v>3229</v>
       </c>
       <c r="Q59" s="28" t="inlineStr">
         <is>
@@ -3833,16 +3833,16 @@
         <v>1146</v>
       </c>
       <c r="I60" s="31" t="n">
-        <v>78</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="J60" s="31" t="n">
-        <v>37247</v>
+        <v>31469</v>
       </c>
       <c r="K60" s="32" t="n">
-        <v>7.3</v>
+        <v>19.5</v>
       </c>
       <c r="L60" s="32" t="n">
-        <v>3486</v>
+        <v>9312</v>
       </c>
       <c r="M60" s="33" t="n">
         <v>12.2</v>
@@ -3851,14 +3851,14 @@
         <v>5826</v>
       </c>
       <c r="O60" s="34" t="n">
-        <v>97.5</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="P60" s="34" t="n">
-        <v>46559</v>
+        <v>46607</v>
       </c>
       <c r="Q60" s="28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -4000,22 +4000,22 @@
         <v>123388</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>62.8</v>
+        <v>60.1</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>77487</v>
+        <v>74156</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>33.4</v>
+        <v>35.5</v>
       </c>
       <c r="K6" s="24" t="n">
-        <v>41211</v>
+        <v>43803</v>
       </c>
       <c r="L6" s="25" t="n">
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="M6" s="25" t="n">
-        <v>4689</v>
+        <v>5429</v>
       </c>
       <c r="N6" s="26" t="n">
         <v>0</v>
@@ -4024,10 +4024,10 @@
         <v>0</v>
       </c>
       <c r="P6" s="27" t="n">
-        <v>37.2</v>
+        <v>39.9</v>
       </c>
       <c r="Q6" s="27" t="n">
-        <v>45900</v>
+        <v>49232</v>
       </c>
       <c r="R6" s="28" t="inlineStr">
         <is>
@@ -4054,10 +4054,10 @@
         <v>11059</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>64.90000000000001</v>
+        <v>64.5</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>7177</v>
+        <v>7133</v>
       </c>
       <c r="J7" s="24" t="n">
         <v>33.2</v>
@@ -4066,10 +4066,10 @@
         <v>3672</v>
       </c>
       <c r="L7" s="25" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="M7" s="25" t="n">
-        <v>210</v>
+        <v>265</v>
       </c>
       <c r="N7" s="26" t="n">
         <v>0</v>
@@ -4078,10 +4078,10 @@
         <v>0</v>
       </c>
       <c r="P7" s="27" t="n">
-        <v>35.1</v>
+        <v>35.6</v>
       </c>
       <c r="Q7" s="27" t="n">
-        <v>3882</v>
+        <v>3937</v>
       </c>
       <c r="R7" s="28" t="inlineStr">
         <is>
@@ -4108,16 +4108,16 @@
         <v>17071</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>66.09999999999999</v>
+        <v>65</v>
       </c>
       <c r="I8" s="23" t="n">
-        <v>11284</v>
+        <v>11096</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>31.8</v>
+        <v>32.8</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>5429</v>
+        <v>5599</v>
       </c>
       <c r="L8" s="25" t="n">
         <v>1.8</v>
@@ -4132,10 +4132,10 @@
         <v>68</v>
       </c>
       <c r="P8" s="27" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q8" s="27" t="n">
-        <v>5804</v>
+        <v>5975</v>
       </c>
       <c r="R8" s="28" t="inlineStr">
         <is>
@@ -4162,22 +4162,22 @@
         <v>15492</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>46.4</v>
+        <v>45.4</v>
       </c>
       <c r="I9" s="23" t="n">
-        <v>7188</v>
+        <v>7033</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>45.9</v>
+        <v>48.1</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>7111</v>
+        <v>7452</v>
       </c>
       <c r="L9" s="25" t="n">
-        <v>5.5</v>
+        <v>4.4</v>
       </c>
       <c r="M9" s="25" t="n">
-        <v>852</v>
+        <v>682</v>
       </c>
       <c r="N9" s="26" t="n">
         <v>2.2</v>
@@ -4186,10 +4186,10 @@
         <v>341</v>
       </c>
       <c r="P9" s="27" t="n">
-        <v>53.6</v>
+        <v>54.7</v>
       </c>
       <c r="Q9" s="27" t="n">
-        <v>8304</v>
+        <v>8474</v>
       </c>
       <c r="R9" s="28" t="inlineStr">
         <is>
@@ -4216,22 +4216,22 @@
         <v>187972</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>38.7</v>
+        <v>37.1</v>
       </c>
       <c r="I10" s="23" t="n">
-        <v>72745</v>
+        <v>69738</v>
       </c>
       <c r="J10" s="24" t="n">
-        <v>55.2</v>
+        <v>54.8</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>103760</v>
+        <v>103009</v>
       </c>
       <c r="L10" s="25" t="n">
-        <v>6</v>
+        <v>8.1</v>
       </c>
       <c r="M10" s="25" t="n">
-        <v>11278</v>
+        <v>15226</v>
       </c>
       <c r="N10" s="26" t="n">
         <v>0</v>
@@ -4240,10 +4240,10 @@
         <v>0</v>
       </c>
       <c r="P10" s="27" t="n">
-        <v>61.2</v>
+        <v>62.9</v>
       </c>
       <c r="Q10" s="27" t="n">
-        <v>115039</v>
+        <v>118234</v>
       </c>
       <c r="R10" s="28" t="inlineStr">
         <is>
@@ -4270,16 +4270,16 @@
         <v>36044</v>
       </c>
       <c r="H11" s="23" t="n">
-        <v>41.3</v>
+        <v>39.8</v>
       </c>
       <c r="I11" s="23" t="n">
-        <v>14886</v>
+        <v>14346</v>
       </c>
       <c r="J11" s="24" t="n">
-        <v>57.2</v>
+        <v>58.7</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>20617</v>
+        <v>21158</v>
       </c>
       <c r="L11" s="25" t="n">
         <v>1</v>
@@ -4294,10 +4294,10 @@
         <v>180</v>
       </c>
       <c r="P11" s="27" t="n">
-        <v>58.7</v>
+        <v>60.2</v>
       </c>
       <c r="Q11" s="27" t="n">
-        <v>21158</v>
+        <v>21699</v>
       </c>
       <c r="R11" s="28" t="inlineStr">
         <is>
@@ -4324,22 +4324,22 @@
         <v>23365</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>62.4</v>
+        <v>60.4</v>
       </c>
       <c r="I12" s="23" t="n">
-        <v>14580</v>
+        <v>14113</v>
       </c>
       <c r="J12" s="24" t="n">
-        <v>34.2</v>
+        <v>36.6</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>7991</v>
+        <v>8552</v>
       </c>
       <c r="L12" s="25" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M12" s="25" t="n">
-        <v>701</v>
+        <v>584</v>
       </c>
       <c r="N12" s="26" t="n">
         <v>0.5</v>
@@ -4348,10 +4348,10 @@
         <v>117</v>
       </c>
       <c r="P12" s="27" t="n">
-        <v>37.7</v>
+        <v>39.6</v>
       </c>
       <c r="Q12" s="27" t="n">
-        <v>8809</v>
+        <v>9253</v>
       </c>
       <c r="R12" s="28" t="inlineStr">
         <is>
@@ -4432,16 +4432,16 @@
         <v>31394</v>
       </c>
       <c r="H14" s="23" t="n">
-        <v>51.9</v>
+        <v>50.9</v>
       </c>
       <c r="I14" s="23" t="n">
-        <v>16293</v>
+        <v>15979</v>
       </c>
       <c r="J14" s="24" t="n">
-        <v>47.6</v>
+        <v>48.6</v>
       </c>
       <c r="K14" s="24" t="n">
-        <v>14943</v>
+        <v>15257</v>
       </c>
       <c r="L14" s="25" t="n">
         <v>0.5</v>
@@ -4456,10 +4456,10 @@
         <v>0</v>
       </c>
       <c r="P14" s="27" t="n">
-        <v>48.1</v>
+        <v>49.1</v>
       </c>
       <c r="Q14" s="27" t="n">
-        <v>15100</v>
+        <v>15414</v>
       </c>
       <c r="R14" s="28" t="inlineStr">
         <is>
@@ -4486,16 +4486,16 @@
         <v>19315</v>
       </c>
       <c r="H15" s="23" t="n">
-        <v>65.7</v>
+        <v>62.2</v>
       </c>
       <c r="I15" s="23" t="n">
-        <v>12690</v>
+        <v>12014</v>
       </c>
       <c r="J15" s="24" t="n">
-        <v>33.6</v>
+        <v>37.1</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>6490</v>
+        <v>7166</v>
       </c>
       <c r="L15" s="25" t="n">
         <v>0.3</v>
@@ -4510,10 +4510,10 @@
         <v>58</v>
       </c>
       <c r="P15" s="27" t="n">
-        <v>34.2</v>
+        <v>37.7</v>
       </c>
       <c r="Q15" s="27" t="n">
-        <v>6606</v>
+        <v>7282</v>
       </c>
       <c r="R15" s="28" t="inlineStr">
         <is>
@@ -4540,16 +4540,16 @@
         <v>32784</v>
       </c>
       <c r="H16" s="23" t="n">
-        <v>54.6</v>
+        <v>47</v>
       </c>
       <c r="I16" s="23" t="n">
-        <v>17900</v>
+        <v>15408</v>
       </c>
       <c r="J16" s="24" t="n">
-        <v>45.4</v>
+        <v>53</v>
       </c>
       <c r="K16" s="24" t="n">
-        <v>14884</v>
+        <v>17375</v>
       </c>
       <c r="L16" s="25" t="n">
         <v>0</v>
@@ -4564,10 +4564,10 @@
         <v>0</v>
       </c>
       <c r="P16" s="27" t="n">
-        <v>45.4</v>
+        <v>53</v>
       </c>
       <c r="Q16" s="27" t="n">
-        <v>14884</v>
+        <v>17375</v>
       </c>
       <c r="R16" s="28" t="inlineStr">
         <is>
@@ -4594,16 +4594,16 @@
         <v>142297</v>
       </c>
       <c r="H17" s="23" t="n">
-        <v>42</v>
+        <v>34.6</v>
       </c>
       <c r="I17" s="23" t="n">
-        <v>59765</v>
+        <v>49235</v>
       </c>
       <c r="J17" s="24" t="n">
-        <v>57.4</v>
+        <v>64.8</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>81678</v>
+        <v>92208</v>
       </c>
       <c r="L17" s="25" t="n">
         <v>0</v>
@@ -4618,10 +4618,10 @@
         <v>854</v>
       </c>
       <c r="P17" s="27" t="n">
-        <v>58</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q17" s="27" t="n">
-        <v>82532</v>
+        <v>93062</v>
       </c>
       <c r="R17" s="28" t="inlineStr">
         <is>
@@ -4648,16 +4648,16 @@
         <v>9550</v>
       </c>
       <c r="H18" s="23" t="n">
-        <v>52</v>
+        <v>45.5</v>
       </c>
       <c r="I18" s="23" t="n">
-        <v>4966</v>
+        <v>4345</v>
       </c>
       <c r="J18" s="24" t="n">
-        <v>47.5</v>
+        <v>54</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>4536</v>
+        <v>5157</v>
       </c>
       <c r="L18" s="25" t="n">
         <v>0</v>
@@ -4672,10 +4672,10 @@
         <v>48</v>
       </c>
       <c r="P18" s="27" t="n">
-        <v>48</v>
+        <v>54.5</v>
       </c>
       <c r="Q18" s="27" t="n">
-        <v>4584</v>
+        <v>5205</v>
       </c>
       <c r="R18" s="28" t="inlineStr">
         <is>
@@ -4702,22 +4702,22 @@
         <v>17619</v>
       </c>
       <c r="H19" s="23" t="n">
-        <v>56.1</v>
+        <v>42.4</v>
       </c>
       <c r="I19" s="23" t="n">
-        <v>9884</v>
+        <v>7471</v>
       </c>
       <c r="J19" s="24" t="n">
-        <v>40.9</v>
+        <v>55.3</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>7206</v>
+        <v>9743</v>
       </c>
       <c r="L19" s="25" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="M19" s="25" t="n">
-        <v>529</v>
+        <v>405</v>
       </c>
       <c r="N19" s="26" t="n">
         <v>0</v>
@@ -4726,10 +4726,10 @@
         <v>0</v>
       </c>
       <c r="P19" s="27" t="n">
-        <v>43.9</v>
+        <v>57.6</v>
       </c>
       <c r="Q19" s="27" t="n">
-        <v>7735</v>
+        <v>10149</v>
       </c>
       <c r="R19" s="28" t="inlineStr">
         <is>
@@ -4756,16 +4756,16 @@
         <v>9184</v>
       </c>
       <c r="H20" s="23" t="n">
-        <v>51.3</v>
+        <v>50.9</v>
       </c>
       <c r="I20" s="23" t="n">
-        <v>4711</v>
+        <v>4674</v>
       </c>
       <c r="J20" s="24" t="n">
-        <v>48.3</v>
+        <v>48.7</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>4436</v>
+        <v>4472</v>
       </c>
       <c r="L20" s="25" t="n">
         <v>0.4</v>
@@ -4780,10 +4780,10 @@
         <v>0</v>
       </c>
       <c r="P20" s="27" t="n">
-        <v>48.7</v>
+        <v>49.1</v>
       </c>
       <c r="Q20" s="27" t="n">
-        <v>4472</v>
+        <v>4509</v>
       </c>
       <c r="R20" s="28" t="inlineStr">
         <is>
@@ -4810,22 +4810,22 @@
         <v>28857</v>
       </c>
       <c r="H21" s="23" t="n">
-        <v>35.2</v>
+        <v>34</v>
       </c>
       <c r="I21" s="23" t="n">
-        <v>10158</v>
+        <v>9811</v>
       </c>
       <c r="J21" s="24" t="n">
-        <v>59.7</v>
+        <v>62.9</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>17228</v>
+        <v>18151</v>
       </c>
       <c r="L21" s="25" t="n">
-        <v>3.8</v>
+        <v>1.9</v>
       </c>
       <c r="M21" s="25" t="n">
-        <v>1097</v>
+        <v>548</v>
       </c>
       <c r="N21" s="26" t="n">
         <v>1.3</v>
@@ -4834,10 +4834,10 @@
         <v>375</v>
       </c>
       <c r="P21" s="27" t="n">
-        <v>64.8</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="Q21" s="27" t="n">
-        <v>18699</v>
+        <v>19074</v>
       </c>
       <c r="R21" s="28" t="inlineStr">
         <is>
@@ -4918,16 +4918,16 @@
         <v>24113</v>
       </c>
       <c r="H23" s="23" t="n">
-        <v>37</v>
+        <v>29.5</v>
       </c>
       <c r="I23" s="23" t="n">
-        <v>8922</v>
+        <v>7113</v>
       </c>
       <c r="J23" s="24" t="n">
-        <v>62.7</v>
+        <v>70.2</v>
       </c>
       <c r="K23" s="24" t="n">
-        <v>15119</v>
+        <v>16927</v>
       </c>
       <c r="L23" s="25" t="n">
         <v>0</v>
@@ -4942,10 +4942,10 @@
         <v>72</v>
       </c>
       <c r="P23" s="27" t="n">
-        <v>63</v>
+        <v>70.5</v>
       </c>
       <c r="Q23" s="27" t="n">
-        <v>15191</v>
+        <v>17000</v>
       </c>
       <c r="R23" s="28" t="inlineStr">
         <is>
@@ -4972,22 +4972,22 @@
         <v>182675</v>
       </c>
       <c r="H24" s="23" t="n">
-        <v>49.5</v>
+        <v>45</v>
       </c>
       <c r="I24" s="23" t="n">
-        <v>90424</v>
+        <v>82204</v>
       </c>
       <c r="J24" s="24" t="n">
-        <v>45.4</v>
+        <v>51.8</v>
       </c>
       <c r="K24" s="24" t="n">
-        <v>82934</v>
+        <v>94626</v>
       </c>
       <c r="L24" s="25" t="n">
-        <v>2.8</v>
+        <v>0.9</v>
       </c>
       <c r="M24" s="25" t="n">
-        <v>5115</v>
+        <v>1644</v>
       </c>
       <c r="N24" s="26" t="n">
         <v>2.3</v>
@@ -4996,10 +4996,10 @@
         <v>4202</v>
       </c>
       <c r="P24" s="27" t="n">
-        <v>50.5</v>
+        <v>55</v>
       </c>
       <c r="Q24" s="27" t="n">
-        <v>92251</v>
+        <v>100471</v>
       </c>
       <c r="R24" s="28" t="inlineStr">
         <is>
@@ -5026,16 +5026,16 @@
         <v>35703</v>
       </c>
       <c r="H25" s="23" t="n">
-        <v>66.59999999999999</v>
+        <v>66</v>
       </c>
       <c r="I25" s="23" t="n">
-        <v>23778</v>
+        <v>23564</v>
       </c>
       <c r="J25" s="24" t="n">
-        <v>32</v>
+        <v>32.6</v>
       </c>
       <c r="K25" s="24" t="n">
-        <v>11425</v>
+        <v>11639</v>
       </c>
       <c r="L25" s="25" t="n">
         <v>1.1</v>
@@ -5050,10 +5050,10 @@
         <v>107</v>
       </c>
       <c r="P25" s="27" t="n">
-        <v>33.4</v>
+        <v>34</v>
       </c>
       <c r="Q25" s="27" t="n">
-        <v>11925</v>
+        <v>12139</v>
       </c>
       <c r="R25" s="28" t="inlineStr">
         <is>
@@ -5080,16 +5080,16 @@
         <v>46864</v>
       </c>
       <c r="H26" s="23" t="n">
-        <v>40.6</v>
+        <v>38.3</v>
       </c>
       <c r="I26" s="23" t="n">
-        <v>19027</v>
+        <v>17949</v>
       </c>
       <c r="J26" s="24" t="n">
-        <v>57.7</v>
+        <v>60</v>
       </c>
       <c r="K26" s="24" t="n">
-        <v>27040</v>
+        <v>28118</v>
       </c>
       <c r="L26" s="25" t="n">
         <v>1.1</v>
@@ -5104,10 +5104,10 @@
         <v>281</v>
       </c>
       <c r="P26" s="27" t="n">
-        <v>59.4</v>
+        <v>61.7</v>
       </c>
       <c r="Q26" s="27" t="n">
-        <v>27837</v>
+        <v>28915</v>
       </c>
       <c r="R26" s="28" t="inlineStr">
         <is>
@@ -5140,16 +5140,16 @@
         <v>17187</v>
       </c>
       <c r="J27" s="24" t="n">
-        <v>54.3</v>
+        <v>54.7</v>
       </c>
       <c r="K27" s="24" t="n">
-        <v>24367</v>
+        <v>24546</v>
       </c>
       <c r="L27" s="25" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="M27" s="25" t="n">
-        <v>3321</v>
+        <v>3141</v>
       </c>
       <c r="N27" s="26" t="n">
         <v>0</v>
@@ -5188,16 +5188,16 @@
         <v>64063</v>
       </c>
       <c r="H28" s="23" t="n">
-        <v>48.6</v>
+        <v>45.2</v>
       </c>
       <c r="I28" s="23" t="n">
-        <v>31134</v>
+        <v>28956</v>
       </c>
       <c r="J28" s="24" t="n">
-        <v>49.2</v>
+        <v>52.5</v>
       </c>
       <c r="K28" s="24" t="n">
-        <v>31519</v>
+        <v>33633</v>
       </c>
       <c r="L28" s="25" t="n">
         <v>0.6</v>
@@ -5212,10 +5212,10 @@
         <v>1089</v>
       </c>
       <c r="P28" s="27" t="n">
-        <v>51.5</v>
+        <v>54.8</v>
       </c>
       <c r="Q28" s="27" t="n">
-        <v>32992</v>
+        <v>35106</v>
       </c>
       <c r="R28" s="28" t="inlineStr">
         <is>
@@ -5242,16 +5242,16 @@
         <v>50364</v>
       </c>
       <c r="H29" s="23" t="n">
-        <v>84.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="I29" s="23" t="n">
-        <v>42608</v>
+        <v>41047</v>
       </c>
       <c r="J29" s="24" t="n">
-        <v>15.4</v>
+        <v>18.5</v>
       </c>
       <c r="K29" s="24" t="n">
-        <v>7756</v>
+        <v>9317</v>
       </c>
       <c r="L29" s="25" t="n">
         <v>0</v>
@@ -5266,10 +5266,10 @@
         <v>0</v>
       </c>
       <c r="P29" s="27" t="n">
-        <v>15.4</v>
+        <v>18.5</v>
       </c>
       <c r="Q29" s="27" t="n">
-        <v>7756</v>
+        <v>9317</v>
       </c>
       <c r="R29" s="28" t="inlineStr">
         <is>
@@ -5296,22 +5296,22 @@
         <v>34105</v>
       </c>
       <c r="H30" s="23" t="n">
-        <v>41.7</v>
+        <v>37.9</v>
       </c>
       <c r="I30" s="23" t="n">
-        <v>14222</v>
+        <v>12926</v>
       </c>
       <c r="J30" s="24" t="n">
-        <v>53.8</v>
+        <v>50.8</v>
       </c>
       <c r="K30" s="24" t="n">
-        <v>18349</v>
+        <v>17325</v>
       </c>
       <c r="L30" s="25" t="n">
-        <v>3.8</v>
+        <v>10.6</v>
       </c>
       <c r="M30" s="25" t="n">
-        <v>1296</v>
+        <v>3615</v>
       </c>
       <c r="N30" s="26" t="n">
         <v>0.8</v>
@@ -5320,10 +5320,10 @@
         <v>273</v>
       </c>
       <c r="P30" s="27" t="n">
-        <v>58.4</v>
+        <v>62.2</v>
       </c>
       <c r="Q30" s="27" t="n">
-        <v>19917</v>
+        <v>21213</v>
       </c>
       <c r="R30" s="28" t="inlineStr">
         <is>
@@ -5350,16 +5350,16 @@
         <v>48711</v>
       </c>
       <c r="H31" s="23" t="n">
-        <v>41.3</v>
+        <v>28.4</v>
       </c>
       <c r="I31" s="23" t="n">
-        <v>20118</v>
+        <v>13834</v>
       </c>
       <c r="J31" s="24" t="n">
-        <v>51.4</v>
+        <v>64.2</v>
       </c>
       <c r="K31" s="24" t="n">
-        <v>25038</v>
+        <v>31273</v>
       </c>
       <c r="L31" s="25" t="n">
         <v>5.5</v>
@@ -5374,10 +5374,10 @@
         <v>877</v>
       </c>
       <c r="P31" s="27" t="n">
-        <v>58.7</v>
+        <v>71.5</v>
       </c>
       <c r="Q31" s="27" t="n">
-        <v>28594</v>
+        <v>34829</v>
       </c>
       <c r="R31" s="28" t="inlineStr">
         <is>
@@ -5404,22 +5404,22 @@
         <v>11508</v>
       </c>
       <c r="H32" s="23" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I32" s="23" t="n">
-        <v>1726</v>
+        <v>1151</v>
       </c>
       <c r="J32" s="24" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="K32" s="24" t="n">
-        <v>8631</v>
+        <v>9782</v>
       </c>
       <c r="L32" s="25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M32" s="25" t="n">
-        <v>575</v>
+        <v>0</v>
       </c>
       <c r="N32" s="26" t="n">
         <v>5</v>
@@ -5428,10 +5428,10 @@
         <v>575</v>
       </c>
       <c r="P32" s="27" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="Q32" s="27" t="n">
-        <v>9782</v>
+        <v>10357</v>
       </c>
       <c r="R32" s="28" t="inlineStr">
         <is>
@@ -5674,22 +5674,22 @@
         <v>638</v>
       </c>
       <c r="H37" s="23" t="n">
-        <v>20.3</v>
+        <v>19.6</v>
       </c>
       <c r="I37" s="23" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="J37" s="24" t="n">
-        <v>78.3</v>
+        <v>79.7</v>
       </c>
       <c r="K37" s="24" t="n">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="L37" s="25" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="M37" s="25" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N37" s="26" t="n">
         <v>0.7</v>
@@ -5698,10 +5698,10 @@
         <v>4</v>
       </c>
       <c r="P37" s="27" t="n">
-        <v>79.7</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="Q37" s="27" t="n">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="R37" s="28" t="inlineStr">
         <is>
@@ -5728,22 +5728,22 @@
         <v>60213</v>
       </c>
       <c r="H38" s="23" t="n">
-        <v>51.9</v>
+        <v>50.8</v>
       </c>
       <c r="I38" s="23" t="n">
-        <v>31250</v>
+        <v>30588</v>
       </c>
       <c r="J38" s="24" t="n">
-        <v>48.1</v>
+        <v>48.9</v>
       </c>
       <c r="K38" s="24" t="n">
-        <v>28962</v>
+        <v>29444</v>
       </c>
       <c r="L38" s="25" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="M38" s="25" t="n">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="N38" s="26" t="n">
         <v>0</v>
@@ -5752,10 +5752,10 @@
         <v>0</v>
       </c>
       <c r="P38" s="27" t="n">
-        <v>48.1</v>
+        <v>49.2</v>
       </c>
       <c r="Q38" s="27" t="n">
-        <v>28962</v>
+        <v>29625</v>
       </c>
       <c r="R38" s="28" t="inlineStr">
         <is>
@@ -5782,16 +5782,16 @@
         <v>67918</v>
       </c>
       <c r="H39" s="23" t="n">
-        <v>12.5</v>
+        <v>7.8</v>
       </c>
       <c r="I39" s="23" t="n">
-        <v>8490</v>
+        <v>5298</v>
       </c>
       <c r="J39" s="24" t="n">
-        <v>78.90000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="K39" s="24" t="n">
-        <v>53587</v>
+        <v>56780</v>
       </c>
       <c r="L39" s="25" t="n">
         <v>3.9</v>
@@ -5806,10 +5806,10 @@
         <v>3192</v>
       </c>
       <c r="P39" s="27" t="n">
-        <v>87.5</v>
+        <v>92.2</v>
       </c>
       <c r="Q39" s="27" t="n">
-        <v>59428</v>
+        <v>62620</v>
       </c>
       <c r="R39" s="28" t="inlineStr">
         <is>
@@ -5836,16 +5836,16 @@
         <v>13582</v>
       </c>
       <c r="H40" s="23" t="n">
-        <v>84.8</v>
+        <v>83.8</v>
       </c>
       <c r="I40" s="23" t="n">
-        <v>11517</v>
+        <v>11381</v>
       </c>
       <c r="J40" s="24" t="n">
-        <v>15.2</v>
+        <v>16.2</v>
       </c>
       <c r="K40" s="24" t="n">
-        <v>2064</v>
+        <v>2200</v>
       </c>
       <c r="L40" s="25" t="n">
         <v>0</v>
@@ -5860,10 +5860,10 @@
         <v>0</v>
       </c>
       <c r="P40" s="27" t="n">
-        <v>15.2</v>
+        <v>16.2</v>
       </c>
       <c r="Q40" s="27" t="n">
-        <v>2064</v>
+        <v>2200</v>
       </c>
       <c r="R40" s="28" t="inlineStr">
         <is>
@@ -5890,22 +5890,22 @@
         <v>29215</v>
       </c>
       <c r="H41" s="23" t="n">
-        <v>36.9</v>
+        <v>36.1</v>
       </c>
       <c r="I41" s="23" t="n">
-        <v>10780</v>
+        <v>10547</v>
       </c>
       <c r="J41" s="24" t="n">
-        <v>60.2</v>
+        <v>60.6</v>
       </c>
       <c r="K41" s="24" t="n">
-        <v>17588</v>
+        <v>17704</v>
       </c>
       <c r="L41" s="25" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="M41" s="25" t="n">
-        <v>234</v>
+        <v>351</v>
       </c>
       <c r="N41" s="26" t="n">
         <v>2.1</v>
@@ -5914,10 +5914,10 @@
         <v>614</v>
       </c>
       <c r="P41" s="27" t="n">
-        <v>63.1</v>
+        <v>63.9</v>
       </c>
       <c r="Q41" s="27" t="n">
-        <v>18435</v>
+        <v>18669</v>
       </c>
       <c r="R41" s="28" t="inlineStr">
         <is>
@@ -5944,22 +5944,22 @@
         <v>42481</v>
       </c>
       <c r="H42" s="23" t="n">
-        <v>48.7</v>
+        <v>17.5</v>
       </c>
       <c r="I42" s="23" t="n">
-        <v>20688</v>
+        <v>7434</v>
       </c>
       <c r="J42" s="24" t="n">
-        <v>48.7</v>
+        <v>80.5</v>
       </c>
       <c r="K42" s="24" t="n">
-        <v>20688</v>
+        <v>34198</v>
       </c>
       <c r="L42" s="25" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="M42" s="25" t="n">
-        <v>552</v>
+        <v>255</v>
       </c>
       <c r="N42" s="26" t="n">
         <v>1.3</v>
@@ -5968,10 +5968,10 @@
         <v>552</v>
       </c>
       <c r="P42" s="27" t="n">
-        <v>51.3</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="Q42" s="27" t="n">
-        <v>21793</v>
+        <v>35005</v>
       </c>
       <c r="R42" s="28" t="inlineStr">
         <is>
@@ -5998,16 +5998,16 @@
         <v>156304</v>
       </c>
       <c r="H43" s="23" t="n">
-        <v>65.40000000000001</v>
+        <v>50.2</v>
       </c>
       <c r="I43" s="23" t="n">
-        <v>102223</v>
+        <v>78465</v>
       </c>
       <c r="J43" s="24" t="n">
-        <v>28.3</v>
+        <v>43.4</v>
       </c>
       <c r="K43" s="24" t="n">
-        <v>44234</v>
+        <v>67836</v>
       </c>
       <c r="L43" s="25" t="n">
         <v>5.4</v>
@@ -6022,10 +6022,10 @@
         <v>1563</v>
       </c>
       <c r="P43" s="27" t="n">
-        <v>34.7</v>
+        <v>49.8</v>
       </c>
       <c r="Q43" s="27" t="n">
-        <v>54237</v>
+        <v>77839</v>
       </c>
       <c r="R43" s="28" t="inlineStr">
         <is>
@@ -6052,16 +6052,16 @@
         <v>38531</v>
       </c>
       <c r="H44" s="23" t="n">
-        <v>4.3</v>
+        <v>3.7</v>
       </c>
       <c r="I44" s="23" t="n">
-        <v>1657</v>
+        <v>1426</v>
       </c>
       <c r="J44" s="24" t="n">
-        <v>86.40000000000001</v>
+        <v>87</v>
       </c>
       <c r="K44" s="24" t="n">
-        <v>33291</v>
+        <v>33522</v>
       </c>
       <c r="L44" s="25" t="n">
         <v>9.300000000000001</v>
@@ -6076,10 +6076,10 @@
         <v>0</v>
       </c>
       <c r="P44" s="27" t="n">
-        <v>95.7</v>
+        <v>96.3</v>
       </c>
       <c r="Q44" s="27" t="n">
-        <v>36874</v>
+        <v>37106</v>
       </c>
       <c r="R44" s="28" t="inlineStr">
         <is>
@@ -6106,16 +6106,16 @@
         <v>26900</v>
       </c>
       <c r="H45" s="23" t="n">
-        <v>44.9</v>
+        <v>44.3</v>
       </c>
       <c r="I45" s="23" t="n">
-        <v>12078</v>
+        <v>11916</v>
       </c>
       <c r="J45" s="24" t="n">
-        <v>37.1</v>
+        <v>37.7</v>
       </c>
       <c r="K45" s="24" t="n">
-        <v>9980</v>
+        <v>10141</v>
       </c>
       <c r="L45" s="25" t="n">
         <v>17.4</v>
@@ -6130,10 +6130,10 @@
         <v>161</v>
       </c>
       <c r="P45" s="27" t="n">
-        <v>55.1</v>
+        <v>55.7</v>
       </c>
       <c r="Q45" s="27" t="n">
-        <v>14822</v>
+        <v>14983</v>
       </c>
       <c r="R45" s="28" t="inlineStr">
         <is>
@@ -6160,16 +6160,16 @@
         <v>24608</v>
       </c>
       <c r="H46" s="23" t="n">
-        <v>67.59999999999999</v>
+        <v>38</v>
       </c>
       <c r="I46" s="23" t="n">
-        <v>16635</v>
+        <v>9351</v>
       </c>
       <c r="J46" s="24" t="n">
-        <v>21.1</v>
+        <v>50.7</v>
       </c>
       <c r="K46" s="24" t="n">
-        <v>5192</v>
+        <v>12476</v>
       </c>
       <c r="L46" s="25" t="n">
         <v>7</v>
@@ -6184,10 +6184,10 @@
         <v>1034</v>
       </c>
       <c r="P46" s="27" t="n">
-        <v>32.3</v>
+        <v>61.9</v>
       </c>
       <c r="Q46" s="27" t="n">
-        <v>7948</v>
+        <v>15233</v>
       </c>
       <c r="R46" s="28" t="inlineStr">
         <is>
@@ -6214,22 +6214,22 @@
         <v>16004</v>
       </c>
       <c r="H47" s="23" t="n">
-        <v>48.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I47" s="23" t="n">
-        <v>7778</v>
+        <v>1472</v>
       </c>
       <c r="J47" s="24" t="n">
-        <v>47.7</v>
+        <v>86.2</v>
       </c>
       <c r="K47" s="24" t="n">
-        <v>7634</v>
+        <v>13795</v>
       </c>
       <c r="L47" s="25" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="M47" s="25" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="N47" s="26" t="n">
         <v>3.7</v>
@@ -6238,10 +6238,10 @@
         <v>592</v>
       </c>
       <c r="P47" s="27" t="n">
-        <v>51.4</v>
+        <v>90.8</v>
       </c>
       <c r="Q47" s="27" t="n">
-        <v>8226</v>
+        <v>14531</v>
       </c>
       <c r="R47" s="28" t="inlineStr">
         <is>
@@ -6268,16 +6268,16 @@
         <v>14254</v>
       </c>
       <c r="H48" s="23" t="n">
-        <v>73</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I48" s="23" t="n">
-        <v>10405</v>
+        <v>10206</v>
       </c>
       <c r="J48" s="24" t="n">
-        <v>27</v>
+        <v>28.4</v>
       </c>
       <c r="K48" s="24" t="n">
-        <v>3849</v>
+        <v>4048</v>
       </c>
       <c r="L48" s="25" t="n">
         <v>0</v>
@@ -6292,10 +6292,10 @@
         <v>0</v>
       </c>
       <c r="P48" s="27" t="n">
-        <v>27</v>
+        <v>28.4</v>
       </c>
       <c r="Q48" s="27" t="n">
-        <v>3849</v>
+        <v>4048</v>
       </c>
       <c r="R48" s="28" t="inlineStr">
         <is>
@@ -6322,22 +6322,22 @@
         <v>17317</v>
       </c>
       <c r="H49" s="23" t="n">
-        <v>13.6</v>
+        <v>4.5</v>
       </c>
       <c r="I49" s="23" t="n">
-        <v>2355</v>
+        <v>779</v>
       </c>
       <c r="J49" s="24" t="n">
-        <v>72.7</v>
+        <v>81.3</v>
       </c>
       <c r="K49" s="24" t="n">
-        <v>12589</v>
+        <v>14078</v>
       </c>
       <c r="L49" s="25" t="n">
-        <v>11.9</v>
+        <v>12.5</v>
       </c>
       <c r="M49" s="25" t="n">
-        <v>2061</v>
+        <v>2165</v>
       </c>
       <c r="N49" s="26" t="n">
         <v>1.7</v>
@@ -6346,10 +6346,10 @@
         <v>294</v>
       </c>
       <c r="P49" s="27" t="n">
-        <v>86.3</v>
+        <v>95.5</v>
       </c>
       <c r="Q49" s="27" t="n">
-        <v>14944</v>
+        <v>16537</v>
       </c>
       <c r="R49" s="28" t="inlineStr">
         <is>
@@ -6376,22 +6376,22 @@
         <v>26103</v>
       </c>
       <c r="H50" s="23" t="n">
-        <v>44.2</v>
+        <v>41.1</v>
       </c>
       <c r="I50" s="23" t="n">
-        <v>11538</v>
+        <v>10728</v>
       </c>
       <c r="J50" s="24" t="n">
-        <v>54.3</v>
+        <v>55</v>
       </c>
       <c r="K50" s="24" t="n">
-        <v>14174</v>
+        <v>14357</v>
       </c>
       <c r="L50" s="25" t="n">
-        <v>0.8</v>
+        <v>3.1</v>
       </c>
       <c r="M50" s="25" t="n">
-        <v>209</v>
+        <v>809</v>
       </c>
       <c r="N50" s="26" t="n">
         <v>0.8</v>
@@ -6400,10 +6400,10 @@
         <v>209</v>
       </c>
       <c r="P50" s="27" t="n">
-        <v>55.9</v>
+        <v>58.9</v>
       </c>
       <c r="Q50" s="27" t="n">
-        <v>14592</v>
+        <v>15375</v>
       </c>
       <c r="R50" s="28" t="inlineStr">
         <is>
@@ -6430,16 +6430,16 @@
         <v>4845</v>
       </c>
       <c r="H51" s="23" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="I51" s="23" t="n">
-        <v>3101</v>
+        <v>2859</v>
       </c>
       <c r="J51" s="24" t="n">
-        <v>33.1</v>
+        <v>38.1</v>
       </c>
       <c r="K51" s="24" t="n">
-        <v>1604</v>
+        <v>1846</v>
       </c>
       <c r="L51" s="25" t="n">
         <v>1.4</v>
@@ -6454,10 +6454,10 @@
         <v>68</v>
       </c>
       <c r="P51" s="27" t="n">
-        <v>35.9</v>
+        <v>40.9</v>
       </c>
       <c r="Q51" s="27" t="n">
-        <v>1739</v>
+        <v>1982</v>
       </c>
       <c r="R51" s="28" t="inlineStr">
         <is>
@@ -6484,16 +6484,16 @@
         <v>9533</v>
       </c>
       <c r="H52" s="23" t="n">
-        <v>27.2</v>
+        <v>20.8</v>
       </c>
       <c r="I52" s="23" t="n">
-        <v>2593</v>
+        <v>1983</v>
       </c>
       <c r="J52" s="24" t="n">
-        <v>54.8</v>
+        <v>61.1</v>
       </c>
       <c r="K52" s="24" t="n">
-        <v>5224</v>
+        <v>5825</v>
       </c>
       <c r="L52" s="25" t="n">
         <v>15.9</v>
@@ -6508,10 +6508,10 @@
         <v>200</v>
       </c>
       <c r="P52" s="27" t="n">
-        <v>72.8</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="Q52" s="27" t="n">
-        <v>6940</v>
+        <v>7541</v>
       </c>
       <c r="R52" s="28" t="inlineStr">
         <is>
@@ -6538,22 +6538,22 @@
         <v>30168</v>
       </c>
       <c r="H53" s="23" t="n">
-        <v>16.4</v>
+        <v>11.6</v>
       </c>
       <c r="I53" s="23" t="n">
-        <v>4948</v>
+        <v>3500</v>
       </c>
       <c r="J53" s="24" t="n">
-        <v>75.40000000000001</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="K53" s="24" t="n">
-        <v>22747</v>
+        <v>21842</v>
       </c>
       <c r="L53" s="25" t="n">
-        <v>7.8</v>
+        <v>15.5</v>
       </c>
       <c r="M53" s="25" t="n">
-        <v>2353</v>
+        <v>4676</v>
       </c>
       <c r="N53" s="26" t="n">
         <v>0.4</v>
@@ -6562,10 +6562,10 @@
         <v>121</v>
       </c>
       <c r="P53" s="27" t="n">
-        <v>83.59999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="Q53" s="27" t="n">
-        <v>25221</v>
+        <v>26639</v>
       </c>
       <c r="R53" s="28" t="inlineStr">
         <is>
@@ -6646,22 +6646,22 @@
         <v>37478</v>
       </c>
       <c r="H55" s="23" t="n">
-        <v>54.5</v>
+        <v>52.5</v>
       </c>
       <c r="I55" s="23" t="n">
-        <v>20426</v>
+        <v>19676</v>
       </c>
       <c r="J55" s="24" t="n">
-        <v>26.3</v>
+        <v>27.3</v>
       </c>
       <c r="K55" s="24" t="n">
-        <v>9857</v>
+        <v>10232</v>
       </c>
       <c r="L55" s="25" t="n">
-        <v>13.1</v>
+        <v>14.1</v>
       </c>
       <c r="M55" s="25" t="n">
-        <v>4910</v>
+        <v>5284</v>
       </c>
       <c r="N55" s="26" t="n">
         <v>6.1</v>
@@ -6670,14 +6670,14 @@
         <v>2286</v>
       </c>
       <c r="P55" s="27" t="n">
-        <v>45.5</v>
+        <v>47.5</v>
       </c>
       <c r="Q55" s="27" t="n">
-        <v>17053</v>
+        <v>17802</v>
       </c>
       <c r="R55" s="28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -6700,16 +6700,16 @@
         <v>52658</v>
       </c>
       <c r="H56" s="23" t="n">
-        <v>86.59999999999999</v>
+        <v>85.8</v>
       </c>
       <c r="I56" s="23" t="n">
-        <v>45602</v>
+        <v>45180</v>
       </c>
       <c r="J56" s="24" t="n">
-        <v>10.7</v>
+        <v>11.5</v>
       </c>
       <c r="K56" s="24" t="n">
-        <v>5634</v>
+        <v>6056</v>
       </c>
       <c r="L56" s="25" t="n">
         <v>2.3</v>
@@ -6724,10 +6724,10 @@
         <v>211</v>
       </c>
       <c r="P56" s="27" t="n">
-        <v>13.4</v>
+        <v>14.2</v>
       </c>
       <c r="Q56" s="27" t="n">
-        <v>7056</v>
+        <v>7477</v>
       </c>
       <c r="R56" s="28" t="inlineStr">
         <is>
@@ -6754,10 +6754,10 @@
         <v>7176</v>
       </c>
       <c r="H57" s="23" t="n">
-        <v>56.7</v>
+        <v>55</v>
       </c>
       <c r="I57" s="23" t="n">
-        <v>4069</v>
+        <v>3947</v>
       </c>
       <c r="J57" s="24" t="n">
         <v>40</v>
@@ -6766,10 +6766,10 @@
         <v>2870</v>
       </c>
       <c r="L57" s="25" t="n">
-        <v>1.7</v>
+        <v>3.3</v>
       </c>
       <c r="M57" s="25" t="n">
-        <v>122</v>
+        <v>237</v>
       </c>
       <c r="N57" s="26" t="n">
         <v>1.7</v>
@@ -6778,10 +6778,10 @@
         <v>122</v>
       </c>
       <c r="P57" s="27" t="n">
-        <v>43.4</v>
+        <v>45</v>
       </c>
       <c r="Q57" s="27" t="n">
-        <v>3114</v>
+        <v>3229</v>
       </c>
       <c r="R57" s="28" t="inlineStr">
         <is>
@@ -6814,16 +6814,16 @@
         <v>1146</v>
       </c>
       <c r="J58" s="24" t="n">
-        <v>78</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="K58" s="24" t="n">
-        <v>37247</v>
+        <v>31469</v>
       </c>
       <c r="L58" s="25" t="n">
-        <v>7.3</v>
+        <v>19.5</v>
       </c>
       <c r="M58" s="25" t="n">
-        <v>3486</v>
+        <v>9312</v>
       </c>
       <c r="N58" s="26" t="n">
         <v>12.2</v>
@@ -6832,14 +6832,14 @@
         <v>5826</v>
       </c>
       <c r="P58" s="27" t="n">
-        <v>97.5</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="Q58" s="27" t="n">
-        <v>46559</v>
+        <v>46607</v>
       </c>
       <c r="R58" s="28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8709,16 +8709,16 @@
         <v>1759</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>21.7</v>
+        <v>21.3</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>76.8</v>
+        <v>77.2</v>
       </c>
       <c r="K6" s="24" t="n">
-        <v>1351</v>
+        <v>1358</v>
       </c>
       <c r="L6" s="25" t="n">
         <v>1.1</v>
@@ -8733,10 +8733,10 @@
         <v>7</v>
       </c>
       <c r="P6" s="27" t="n">
-        <v>78.3</v>
+        <v>78.7</v>
       </c>
       <c r="Q6" s="27" t="n">
-        <v>1377</v>
+        <v>1384</v>
       </c>
       <c r="R6" s="28" t="inlineStr">
         <is>
@@ -8763,16 +8763,16 @@
         <v>423</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>49.3</v>
+        <v>48.1</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="J7" s="24" t="n">
-        <v>47</v>
+        <v>48.1</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="L7" s="25" t="n">
         <v>3.4</v>
@@ -8787,10 +8787,10 @@
         <v>2</v>
       </c>
       <c r="P7" s="27" t="n">
-        <v>50.8</v>
+        <v>51.9</v>
       </c>
       <c r="Q7" s="27" t="n">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="R7" s="28" t="inlineStr">
         <is>
@@ -8817,16 +8817,16 @@
         <v>6989</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>29.4</v>
+        <v>24.5</v>
       </c>
       <c r="I8" s="23" t="n">
-        <v>2055</v>
+        <v>1712</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>69.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>4829</v>
+        <v>5172</v>
       </c>
       <c r="L8" s="25" t="n">
         <v>1.3</v>
@@ -8841,10 +8841,10 @@
         <v>21</v>
       </c>
       <c r="P8" s="27" t="n">
-        <v>70.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="Q8" s="27" t="n">
-        <v>4941</v>
+        <v>5284</v>
       </c>
       <c r="R8" s="28" t="inlineStr">
         <is>
@@ -8871,22 +8871,22 @@
         <v>2560</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>29.4</v>
+        <v>28.7</v>
       </c>
       <c r="I9" s="23" t="n">
-        <v>753</v>
+        <v>735</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>60.5</v>
+        <v>60.8</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>1549</v>
+        <v>1556</v>
       </c>
       <c r="L9" s="25" t="n">
-        <v>9.1</v>
+        <v>9.5</v>
       </c>
       <c r="M9" s="25" t="n">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="N9" s="26" t="n">
         <v>1</v>
@@ -8895,10 +8895,10 @@
         <v>26</v>
       </c>
       <c r="P9" s="27" t="n">
-        <v>70.59999999999999</v>
+        <v>71.3</v>
       </c>
       <c r="Q9" s="27" t="n">
-        <v>1807</v>
+        <v>1825</v>
       </c>
       <c r="R9" s="28" t="inlineStr">
         <is>
@@ -8925,16 +8925,16 @@
         <v>3884</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>20.2</v>
+        <v>19.9</v>
       </c>
       <c r="I10" s="23" t="n">
-        <v>785</v>
+        <v>773</v>
       </c>
       <c r="J10" s="24" t="n">
-        <v>79.5</v>
+        <v>79.8</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>3088</v>
+        <v>3099</v>
       </c>
       <c r="L10" s="25" t="n">
         <v>0.3</v>
@@ -8949,10 +8949,10 @@
         <v>0</v>
       </c>
       <c r="P10" s="27" t="n">
-        <v>79.8</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="Q10" s="27" t="n">
-        <v>3099</v>
+        <v>3111</v>
       </c>
       <c r="R10" s="28" t="inlineStr">
         <is>
@@ -8979,16 +8979,16 @@
         <v>11678</v>
       </c>
       <c r="H11" s="23" t="n">
-        <v>52.6</v>
+        <v>51.3</v>
       </c>
       <c r="I11" s="23" t="n">
-        <v>6143</v>
+        <v>5991</v>
       </c>
       <c r="J11" s="24" t="n">
-        <v>45.7</v>
+        <v>47.1</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>5337</v>
+        <v>5500</v>
       </c>
       <c r="L11" s="25" t="n">
         <v>1.7</v>
@@ -9003,10 +9003,10 @@
         <v>0</v>
       </c>
       <c r="P11" s="27" t="n">
-        <v>47.4</v>
+        <v>48.8</v>
       </c>
       <c r="Q11" s="27" t="n">
-        <v>5535</v>
+        <v>5699</v>
       </c>
       <c r="R11" s="28" t="inlineStr">
         <is>
@@ -9033,16 +9033,16 @@
         <v>1518</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>51.2</v>
+        <v>49</v>
       </c>
       <c r="I12" s="23" t="n">
-        <v>777</v>
+        <v>744</v>
       </c>
       <c r="J12" s="24" t="n">
-        <v>46.2</v>
+        <v>48.3</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>701</v>
+        <v>733</v>
       </c>
       <c r="L12" s="25" t="n">
         <v>2.2</v>
@@ -9057,10 +9057,10 @@
         <v>8</v>
       </c>
       <c r="P12" s="27" t="n">
-        <v>48.9</v>
+        <v>51</v>
       </c>
       <c r="Q12" s="27" t="n">
-        <v>742</v>
+        <v>774</v>
       </c>
       <c r="R12" s="28" t="inlineStr">
         <is>
@@ -9087,16 +9087,16 @@
         <v>63</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>74.7</v>
+        <v>73.7</v>
       </c>
       <c r="I13" s="23" t="n">
         <v>47</v>
       </c>
       <c r="J13" s="24" t="n">
-        <v>25.3</v>
+        <v>26.3</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L13" s="25" t="n">
         <v>0</v>
@@ -9111,10 +9111,10 @@
         <v>0</v>
       </c>
       <c r="P13" s="27" t="n">
-        <v>25.3</v>
+        <v>26.3</v>
       </c>
       <c r="Q13" s="27" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R13" s="28" t="inlineStr">
         <is>
@@ -9147,16 +9147,16 @@
         <v>221</v>
       </c>
       <c r="J14" s="24" t="n">
-        <v>54.9</v>
+        <v>54.5</v>
       </c>
       <c r="K14" s="24" t="n">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="L14" s="25" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="M14" s="25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N14" s="26" t="n">
         <v>0</v>
@@ -9165,10 +9165,10 @@
         <v>0</v>
       </c>
       <c r="P14" s="27" t="n">
-        <v>54.9</v>
+        <v>54.8</v>
       </c>
       <c r="Q14" s="27" t="n">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="R14" s="28" t="inlineStr">
         <is>
@@ -9195,16 +9195,16 @@
         <v>1505</v>
       </c>
       <c r="H15" s="23" t="n">
-        <v>71.59999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="I15" s="23" t="n">
-        <v>1078</v>
+        <v>1061</v>
       </c>
       <c r="J15" s="24" t="n">
-        <v>27.9</v>
+        <v>29.1</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>420</v>
+        <v>438</v>
       </c>
       <c r="L15" s="25" t="n">
         <v>0</v>
@@ -9219,10 +9219,10 @@
         <v>8</v>
       </c>
       <c r="P15" s="27" t="n">
-        <v>28.4</v>
+        <v>29.6</v>
       </c>
       <c r="Q15" s="27" t="n">
-        <v>427</v>
+        <v>445</v>
       </c>
       <c r="R15" s="28" t="inlineStr">
         <is>
@@ -9249,16 +9249,16 @@
         <v>187</v>
       </c>
       <c r="H16" s="23" t="n">
-        <v>56.8</v>
+        <v>53.6</v>
       </c>
       <c r="I16" s="23" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="J16" s="24" t="n">
-        <v>41.5</v>
+        <v>44.8</v>
       </c>
       <c r="K16" s="24" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="L16" s="25" t="n">
         <v>0.3</v>
@@ -9273,10 +9273,10 @@
         <v>3</v>
       </c>
       <c r="P16" s="27" t="n">
-        <v>43.2</v>
+        <v>46.5</v>
       </c>
       <c r="Q16" s="27" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="R16" s="28" t="inlineStr">
         <is>
@@ -9303,22 +9303,22 @@
         <v>19148</v>
       </c>
       <c r="H17" s="23" t="n">
-        <v>31.4</v>
+        <v>23.9</v>
       </c>
       <c r="I17" s="23" t="n">
-        <v>6012</v>
+        <v>4576</v>
       </c>
       <c r="J17" s="24" t="n">
-        <v>54</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>10340</v>
+        <v>12274</v>
       </c>
       <c r="L17" s="25" t="n">
-        <v>12</v>
+        <v>9.4</v>
       </c>
       <c r="M17" s="25" t="n">
-        <v>2298</v>
+        <v>1800</v>
       </c>
       <c r="N17" s="26" t="n">
         <v>2.6</v>
@@ -9327,10 +9327,10 @@
         <v>498</v>
       </c>
       <c r="P17" s="27" t="n">
-        <v>68.59999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="Q17" s="27" t="n">
-        <v>13135</v>
+        <v>14572</v>
       </c>
       <c r="R17" s="28" t="inlineStr">
         <is>
@@ -9363,16 +9363,16 @@
         <v>197</v>
       </c>
       <c r="J18" s="24" t="n">
-        <v>78.59999999999999</v>
+        <v>53.6</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>4296</v>
+        <v>2930</v>
       </c>
       <c r="L18" s="25" t="n">
-        <v>3.6</v>
+        <v>28.6</v>
       </c>
       <c r="M18" s="25" t="n">
-        <v>197</v>
+        <v>1563</v>
       </c>
       <c r="N18" s="26" t="n">
         <v>14.3</v>
@@ -9388,7 +9388,7 @@
       </c>
       <c r="R18" s="28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -9411,16 +9411,16 @@
         <v>383</v>
       </c>
       <c r="H19" s="23" t="n">
-        <v>3.7</v>
+        <v>2.8</v>
       </c>
       <c r="I19" s="23" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J19" s="24" t="n">
-        <v>96.3</v>
+        <v>97.2</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="L19" s="25" t="n">
         <v>0</v>
@@ -9435,10 +9435,10 @@
         <v>0</v>
       </c>
       <c r="P19" s="27" t="n">
-        <v>96.3</v>
+        <v>97.2</v>
       </c>
       <c r="Q19" s="27" t="n">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="R19" s="28" t="inlineStr">
         <is>
@@ -9465,16 +9465,16 @@
         <v>23519</v>
       </c>
       <c r="H20" s="23" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="I20" s="23" t="n">
-        <v>141</v>
+        <v>71</v>
       </c>
       <c r="J20" s="24" t="n">
-        <v>98.3</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>23119</v>
+        <v>23189</v>
       </c>
       <c r="L20" s="25" t="n">
         <v>0.6</v>
@@ -9489,10 +9489,10 @@
         <v>141</v>
       </c>
       <c r="P20" s="27" t="n">
-        <v>99.5</v>
+        <v>99.8</v>
       </c>
       <c r="Q20" s="27" t="n">
-        <v>23401</v>
+        <v>23472</v>
       </c>
       <c r="R20" s="28" t="inlineStr">
         <is>
@@ -9519,16 +9519,16 @@
         <v>10543</v>
       </c>
       <c r="H21" s="23" t="n">
-        <v>34.1</v>
+        <v>33</v>
       </c>
       <c r="I21" s="23" t="n">
-        <v>3595</v>
+        <v>3479</v>
       </c>
       <c r="J21" s="24" t="n">
-        <v>59.1</v>
+        <v>60.2</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>6231</v>
+        <v>6347</v>
       </c>
       <c r="L21" s="25" t="n">
         <v>2.3</v>
@@ -9543,10 +9543,10 @@
         <v>474</v>
       </c>
       <c r="P21" s="27" t="n">
-        <v>65.90000000000001</v>
+        <v>67</v>
       </c>
       <c r="Q21" s="27" t="n">
-        <v>6948</v>
+        <v>7064</v>
       </c>
       <c r="R21" s="28" t="inlineStr">
         <is>
@@ -9573,16 +9573,16 @@
         <v>43</v>
       </c>
       <c r="H22" s="23" t="n">
-        <v>7.8</v>
+        <v>6.3</v>
       </c>
       <c r="I22" s="23" t="n">
         <v>3</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>91.90000000000001</v>
+        <v>93.5</v>
       </c>
       <c r="K22" s="24" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L22" s="25" t="n">
         <v>0</v>
@@ -9597,10 +9597,10 @@
         <v>0</v>
       </c>
       <c r="P22" s="27" t="n">
-        <v>92.2</v>
+        <v>93.8</v>
       </c>
       <c r="Q22" s="27" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="R22" s="28" t="inlineStr">
         <is>
@@ -9627,16 +9627,16 @@
         <v>6247</v>
       </c>
       <c r="H23" s="23" t="n">
-        <v>5.8</v>
+        <v>4.7</v>
       </c>
       <c r="I23" s="23" t="n">
-        <v>362</v>
+        <v>294</v>
       </c>
       <c r="J23" s="24" t="n">
-        <v>89.5</v>
+        <v>90.7</v>
       </c>
       <c r="K23" s="24" t="n">
-        <v>5591</v>
+        <v>5666</v>
       </c>
       <c r="L23" s="25" t="n">
         <v>1.6</v>
@@ -9651,10 +9651,10 @@
         <v>194</v>
       </c>
       <c r="P23" s="27" t="n">
-        <v>94.2</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="Q23" s="27" t="n">
-        <v>5885</v>
+        <v>5960</v>
       </c>
       <c r="R23" s="28" t="inlineStr">
         <is>
@@ -9681,13 +9681,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="23" t="n">
-        <v>52.7</v>
+        <v>52.6</v>
       </c>
       <c r="I24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="24" t="n">
-        <v>38.1</v>
+        <v>38.2</v>
       </c>
       <c r="K24" s="24" t="n">
         <v>0</v>
@@ -9705,7 +9705,7 @@
         <v>0</v>
       </c>
       <c r="P24" s="27" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="Q24" s="27" t="n">
         <v>0</v>
@@ -9735,16 +9735,16 @@
         <v>191</v>
       </c>
       <c r="H25" s="23" t="n">
-        <v>49.7</v>
+        <v>27.8</v>
       </c>
       <c r="I25" s="23" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="J25" s="24" t="n">
-        <v>18.7</v>
+        <v>40.6</v>
       </c>
       <c r="K25" s="24" t="n">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="L25" s="25" t="n">
         <v>29.4</v>
@@ -9759,10 +9759,10 @@
         <v>4</v>
       </c>
       <c r="P25" s="27" t="n">
-        <v>50.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="Q25" s="27" t="n">
-        <v>96</v>
+        <v>138</v>
       </c>
       <c r="R25" s="28" t="inlineStr">
         <is>
@@ -9789,22 +9789,22 @@
         <v>19897</v>
       </c>
       <c r="H26" s="23" t="n">
-        <v>50.8</v>
+        <v>30.9</v>
       </c>
       <c r="I26" s="23" t="n">
-        <v>10108</v>
+        <v>6148</v>
       </c>
       <c r="J26" s="24" t="n">
-        <v>36.6</v>
+        <v>56.9</v>
       </c>
       <c r="K26" s="24" t="n">
-        <v>7282</v>
+        <v>11322</v>
       </c>
       <c r="L26" s="25" t="n">
-        <v>10.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M26" s="25" t="n">
-        <v>2030</v>
+        <v>1950</v>
       </c>
       <c r="N26" s="26" t="n">
         <v>2.4</v>
@@ -9813,10 +9813,10 @@
         <v>478</v>
       </c>
       <c r="P26" s="27" t="n">
-        <v>49.2</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="Q26" s="27" t="n">
-        <v>9789</v>
+        <v>13749</v>
       </c>
       <c r="R26" s="28" t="inlineStr">
         <is>
@@ -9897,16 +9897,16 @@
         <v>9197</v>
       </c>
       <c r="H28" s="23" t="n">
-        <v>42.1</v>
+        <v>39</v>
       </c>
       <c r="I28" s="23" t="n">
-        <v>3872</v>
+        <v>3587</v>
       </c>
       <c r="J28" s="24" t="n">
-        <v>36.4</v>
+        <v>39.5</v>
       </c>
       <c r="K28" s="24" t="n">
-        <v>3348</v>
+        <v>3633</v>
       </c>
       <c r="L28" s="25" t="n">
         <v>21</v>
@@ -9921,10 +9921,10 @@
         <v>46</v>
       </c>
       <c r="P28" s="27" t="n">
-        <v>57.9</v>
+        <v>61</v>
       </c>
       <c r="Q28" s="27" t="n">
-        <v>5325</v>
+        <v>5610</v>
       </c>
       <c r="R28" s="28" t="inlineStr">
         <is>
@@ -9957,16 +9957,16 @@
         <v>491</v>
       </c>
       <c r="J29" s="24" t="n">
-        <v>22.3</v>
+        <v>23</v>
       </c>
       <c r="K29" s="24" t="n">
-        <v>1386</v>
+        <v>1429</v>
       </c>
       <c r="L29" s="25" t="n">
-        <v>66.2</v>
+        <v>65.5</v>
       </c>
       <c r="M29" s="25" t="n">
-        <v>4114</v>
+        <v>4071</v>
       </c>
       <c r="N29" s="26" t="n">
         <v>3.6</v>
@@ -10005,16 +10005,16 @@
         <v>3184</v>
       </c>
       <c r="H30" s="23" t="n">
-        <v>65.5</v>
+        <v>54.3</v>
       </c>
       <c r="I30" s="23" t="n">
-        <v>2085</v>
+        <v>1729</v>
       </c>
       <c r="J30" s="24" t="n">
-        <v>32.8</v>
+        <v>44</v>
       </c>
       <c r="K30" s="24" t="n">
-        <v>1044</v>
+        <v>1401</v>
       </c>
       <c r="L30" s="25" t="n">
         <v>1.7</v>
@@ -10029,10 +10029,10 @@
         <v>0</v>
       </c>
       <c r="P30" s="27" t="n">
-        <v>34.5</v>
+        <v>45.7</v>
       </c>
       <c r="Q30" s="27" t="n">
-        <v>1098</v>
+        <v>1455</v>
       </c>
       <c r="R30" s="28" t="inlineStr">
         <is>
@@ -10059,22 +10059,22 @@
         <v>1515</v>
       </c>
       <c r="H31" s="23" t="n">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="I31" s="23" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="J31" s="24" t="n">
-        <v>56.4</v>
+        <v>67.3</v>
       </c>
       <c r="K31" s="24" t="n">
-        <v>855</v>
+        <v>1020</v>
       </c>
       <c r="L31" s="25" t="n">
-        <v>20.9</v>
+        <v>24.5</v>
       </c>
       <c r="M31" s="25" t="n">
-        <v>317</v>
+        <v>371</v>
       </c>
       <c r="N31" s="26" t="n">
         <v>8.199999999999999</v>
@@ -10083,10 +10083,10 @@
         <v>124</v>
       </c>
       <c r="P31" s="27" t="n">
-        <v>85.5</v>
+        <v>100</v>
       </c>
       <c r="Q31" s="27" t="n">
-        <v>1296</v>
+        <v>1515</v>
       </c>
       <c r="R31" s="28" t="inlineStr">
         <is>
@@ -10113,22 +10113,22 @@
         <v>11328</v>
       </c>
       <c r="H32" s="23" t="n">
-        <v>27.8</v>
+        <v>24.3</v>
       </c>
       <c r="I32" s="23" t="n">
-        <v>3149</v>
+        <v>2753</v>
       </c>
       <c r="J32" s="24" t="n">
-        <v>67.40000000000001</v>
+        <v>70.3</v>
       </c>
       <c r="K32" s="24" t="n">
-        <v>7635</v>
+        <v>7964</v>
       </c>
       <c r="L32" s="25" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
       <c r="M32" s="25" t="n">
-        <v>476</v>
+        <v>544</v>
       </c>
       <c r="N32" s="26" t="n">
         <v>0.6</v>
@@ -10137,10 +10137,10 @@
         <v>68</v>
       </c>
       <c r="P32" s="27" t="n">
-        <v>72.2</v>
+        <v>75.7</v>
       </c>
       <c r="Q32" s="27" t="n">
-        <v>8179</v>
+        <v>8575</v>
       </c>
       <c r="R32" s="28" t="inlineStr">
         <is>
@@ -10167,16 +10167,16 @@
         <v>13858</v>
       </c>
       <c r="H33" s="23" t="n">
-        <v>44.4</v>
+        <v>37.9</v>
       </c>
       <c r="I33" s="23" t="n">
-        <v>6153</v>
+        <v>5252</v>
       </c>
       <c r="J33" s="24" t="n">
-        <v>46.8</v>
+        <v>53.2</v>
       </c>
       <c r="K33" s="24" t="n">
-        <v>6486</v>
+        <v>7373</v>
       </c>
       <c r="L33" s="25" t="n">
         <v>5.2</v>
@@ -10191,10 +10191,10 @@
         <v>499</v>
       </c>
       <c r="P33" s="27" t="n">
-        <v>55.6</v>
+        <v>62</v>
       </c>
       <c r="Q33" s="27" t="n">
-        <v>7705</v>
+        <v>8592</v>
       </c>
       <c r="R33" s="28" t="inlineStr">
         <is>
@@ -10221,16 +10221,16 @@
         <v>316</v>
       </c>
       <c r="H34" s="23" t="n">
-        <v>22.6</v>
+        <v>15.7</v>
       </c>
       <c r="I34" s="23" t="n">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="J34" s="24" t="n">
-        <v>55.3</v>
+        <v>62.2</v>
       </c>
       <c r="K34" s="24" t="n">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="L34" s="25" t="n">
         <v>21.2</v>
@@ -10245,10 +10245,10 @@
         <v>3</v>
       </c>
       <c r="P34" s="27" t="n">
-        <v>77.40000000000001</v>
+        <v>84.3</v>
       </c>
       <c r="Q34" s="27" t="n">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="R34" s="28" t="inlineStr">
         <is>
@@ -10275,16 +10275,16 @@
         <v>18724</v>
       </c>
       <c r="H35" s="23" t="n">
-        <v>19.3</v>
+        <v>17.4</v>
       </c>
       <c r="I35" s="23" t="n">
-        <v>3614</v>
+        <v>3258</v>
       </c>
       <c r="J35" s="24" t="n">
-        <v>78.8</v>
+        <v>80.7</v>
       </c>
       <c r="K35" s="24" t="n">
-        <v>14754</v>
+        <v>15110</v>
       </c>
       <c r="L35" s="25" t="n">
         <v>1.5</v>
@@ -10299,10 +10299,10 @@
         <v>75</v>
       </c>
       <c r="P35" s="27" t="n">
-        <v>80.7</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="Q35" s="27" t="n">
-        <v>15110</v>
+        <v>15466</v>
       </c>
       <c r="R35" s="28" t="inlineStr">
         <is>
@@ -10329,22 +10329,22 @@
         <v>6746</v>
       </c>
       <c r="H36" s="23" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I36" s="23" t="n">
-        <v>1552</v>
+        <v>1417</v>
       </c>
       <c r="J36" s="24" t="n">
-        <v>57.6</v>
+        <v>60</v>
       </c>
       <c r="K36" s="24" t="n">
-        <v>3885</v>
+        <v>4047</v>
       </c>
       <c r="L36" s="25" t="n">
-        <v>17.5</v>
+        <v>17.2</v>
       </c>
       <c r="M36" s="25" t="n">
-        <v>1180</v>
+        <v>1160</v>
       </c>
       <c r="N36" s="26" t="n">
         <v>1.9</v>
@@ -10353,10 +10353,10 @@
         <v>128</v>
       </c>
       <c r="P36" s="27" t="n">
-        <v>77</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="Q36" s="27" t="n">
-        <v>5194</v>
+        <v>5336</v>
       </c>
       <c r="R36" s="28" t="inlineStr">
         <is>
@@ -10383,22 +10383,22 @@
         <v>4821</v>
       </c>
       <c r="H37" s="23" t="n">
-        <v>10.1</v>
+        <v>2.3</v>
       </c>
       <c r="I37" s="23" t="n">
-        <v>487</v>
+        <v>111</v>
       </c>
       <c r="J37" s="24" t="n">
-        <v>66.09999999999999</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="K37" s="24" t="n">
-        <v>3187</v>
+        <v>3548</v>
       </c>
       <c r="L37" s="25" t="n">
-        <v>22.5</v>
+        <v>22.8</v>
       </c>
       <c r="M37" s="25" t="n">
-        <v>1085</v>
+        <v>1099</v>
       </c>
       <c r="N37" s="26" t="n">
         <v>1.3</v>
@@ -10407,10 +10407,10 @@
         <v>63</v>
       </c>
       <c r="P37" s="27" t="n">
-        <v>89.90000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="Q37" s="27" t="n">
-        <v>4334</v>
+        <v>4710</v>
       </c>
       <c r="R37" s="28" t="inlineStr">
         <is>

</xml_diff>